<commit_message>
Update berita 2026-08-05 21:05 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,13 +419,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -1655,8 +1655,102 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Madrid dan Leipzig Sepakati Transfer Diomande, Nilainya Segini</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 02:00:05 +0700</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Mohammad Resha Pratama</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Real Madrid akhirnya mencapai kata sepakat dengan RB Leipzig soal transfer Yan Diomande. Winger Pantai Gading itu selangkah lagi berseragam putih-putih.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8606221/madrid-dan-leipzig-sepakati-transfer-diomande-nilainya-segini</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/yan-diomande-1785952593058_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Tanpa Penonton, Final Piala Presiden Tetap Dijaga Ketat Aparat</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 01:00:15 +0700</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Muhammad Robbani</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Organizing Committee (OC) Piala Presiden 2026 Arya Sinulingga ungkap alasan final tanpa penonton. Tanpa penonton, laga tetap dijaga ketat aparat.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8606219/tanpa-penonton-final-piala-presiden-tetap-dijaga-ketat-aparat</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/06/ilustrasi-logo-piala-presiden-2026-1783328492093_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I26"/>
+  <autoFilter ref="A1:I28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-05 22:14 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1749,8 +1749,714 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Arsenal sepakat datangkan Bruno Guimaraes</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:52:58 +0700</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Juara Liga Inggris Arsenal dilaporkan mencapai kesepakatan untuk mendatangkan gelandang Newcastle United Bruno ...</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681809/arsenal-sepakat-datangkan-bruno-guimaraes</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/05/19/2023-05-18T204216Z_664206330_UP1EJ5I1LIETK_RTRMADP_3_SOCCER-ENGLAND-NEW-BRH-REPORT.jpg</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Mohamed Salah gabung Trabzonspor</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:47:52 +0700</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Mohamed Salah bergabung dengan klub Turki Trabzonspor setelah didatangkan dari Liverpool dalam status bebas ...</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681808/mohamed-salah-gabung-trabzonspor</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/04/XxjpseE000147_20260704_PEPFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Newcastle tunjuk Matthias Jaissle sebagai pelatih kepala baru</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:43:37 +0700</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Newcastle United  menunjuk Matthias Jaissle sebagai pelatih kepala baru menggantikan Eddie Howe yang mundur ...</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681807/newcastle-tunjuk-matthias-jaissle-sebagai-pelatih-kepala-baru</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/11/12/ilustrasi-newcastle.jpg</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Perputaran ekonomi Piala Presiden 2026 capai Rp1,5 miliar</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:37:14 +0700</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Ketua Organizing Committee (OC) Piala Presiden 2026 Tsamara Amany mengungkapkan total perputaran ekonomi turnamen ...</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681804/perputaran-ekonomi-piala-presiden-2026-capai-rp15-miliar</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG-20260806-WA0002.jpg</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Luis Figo desak Presiden FIFA Gianni Infantino mundur</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:30:38 +0700</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Gelandang legendaris Portugal, Luis Figo, mendesak Presiden FIFA Gianni Infantino mundur.
+"Hari ini, saya ...</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681803/luis-figo-desak-presiden-fifa-gianni-infantino-mundur</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/12/IMG-20260712-WA0131.jpg</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Undana bentuk tim investigasi soal kasus mahasiswi depresi</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ANTARA - Universitas Nusa Cendana membentuk tim investigasi sebagai tindak lanjut atas kasus yang menimpa mahasiswi ...</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681787/undana-bentuk-tim-investigasi-soal-kasus-mahasiswi-depresi</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_UNDANA-BENTUK-TIM-INVESTIGASI.jpg</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Zhergova antar Juventus taklukkan Chelsea 1-0</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:26:06 +0700</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Edon Zhergova mengantarkan Juventus menaklukkan Chelsea 1-0 pada pertandingan persahabatan di Stadion Kai Tak Sports ...</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681799/zhergova-antar-juventus-taklukkan-chelsea-1-0</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2022/10/30/1667073098700.jpg</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Derby Milano di Perth berakhir imbang 1-1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:20:11 +0700</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Derby Milano antara AC Milan dan Inter Milan berakhir imbang 1-1 pada pertandingan persahabatan di Stadion Optus, ...</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681796/derby-milano-di-perth-berakhir-imbang-1-1</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/2026.jpg</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Manchester City tekuk K-League All Stars 3-1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:15:21 +0700</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Manchester City mengandaskan tim K-League All Stars dengan  3-1 pada pertandingan persahabatan di Stadion Seoul ...</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681792/manchester-city-tekuk-k-league-all-stars-3-1</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/semenyo.jpg</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Diupah Rp 100 Ribu, Pemulung di Makassar Bantu Angkut Kabel BTS Hasil Curian</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 05:00:16 +0700</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Reinhard Soplantila</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Polisi menangkap SA, pria 38 tahun, yang terlibat pencurian kabel BTS di Makassar. Ia mengaku dibayar Rp 100 ribu untuk membantu mengangkut barang curian.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606265/diupah-rp-100-ribu-pemulung-di-makassar-bantu-angkut-kabel-bts-hasil-curian</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/polisi-menangkap-pria-berinisial-sa-terkait-kasus-pencurian-kabel-dan-perlengkapan-menara-bts-1785935325035_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Pemerintah Nigeria Bebaskan 308 Korban Penculikan Bandit-Kelompok Jihadis</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 04:33:36 +0700</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Farih Maulana Sidik</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Pemerintah Nigeria berhasil membebaskan 308 warga yang diculik, termasuk 163 dari Desa Woro. Penculikan ini menjadi krisis besar di negara tersebut.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606261/pemerintah-nigeria-bebaskan-308-korban-penculikan-bandit-kelompok-jihadis</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/11/21/personel-militer-nigeria-berpatroli-di-lokasi-serangan-militan-1763722354741_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>AS Cabut Sanksi Maskapai Irak yang Terkait Garda Revolusi Iran</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 03:55:57 +0700</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Farih Maulana Sidik</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>AS mencabut sanksi terhadap maskapai Fly Baghdad setelah peninjauan. Namun, sanksi terhadap pemiliknya tetap berlaku. Perubahan operasional jadi faktor utama.</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606259/as-cabut-sanksi-maskapai-irak-yang-terkait-garda-revolusi-iran</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/14/ilustrasi-pesawat_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Gempa M 5,4 Guncang Boven Digoel Papua</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 03:08:50 +0700</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Farih Maulana Sidik</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Gempa bumi magnitudo 5,4 mengguncang Kabupaten Boven Digoel, Papua Selatan, pada kedalaman 57 km. BMKG menginformasikan gempa terjadi pukul 02.46 WIB.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606256/gempa-m-5-4-guncang-boven-digoel-papua</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/08/ilustrasi-gempa-1780909642348_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Bocah di Jambi Tewas Diterkam Buaya Saat Mandi di Sungai</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 03:00:31 +0700</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Dimas Sanjaya</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Seorang bocah 11 tahun, M Dzaki, tewas diterkam buaya saat mandi di sungai di Jambi. Temannya, Aldi, mengalami luka dan dirawat.</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606255/bocah-di-jambi-tewas-diterkam-buaya-saat-mandi-di-sungai</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/petugas-saat-mengevakuasi-bocah-yang-tewas-diterkam-buaya-1785899635913_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Pasutri di Bandung Kompak Jadi Jambret, Motifnya Masalah Ekonomi</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 02:33:33 +0700</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Wisma Putra</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Pasangan suami-istri di Bandung ditangkap setelah menjambret handphone anak di bawah umur. Motifnya diduga karena masalah ekonomi. Terancam 9 tahun penjara.</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606249/pasutri-di-bandung-kompak-jadi-jambret-motifnya-masalah-ekonomi</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2015/11/13/366624f0-eb8f-4197-9ef1-fab9055cc0dc_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I28"/>
+  <autoFilter ref="A1:I43"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-05 23:53 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,10 +419,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
@@ -2455,8 +2455,756 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Darwinbox Luncurkan Cortex, Platform HCM AI-Native Terbaru</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:42:06 +0700</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>- Darwinbox adalah platform Human Capital Management yang terkemuka di dunia dan melayani lebih dari 1.400 perusahaan ...</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681844/darwinbox-luncurkan-cortex-platform-hcm-ai-native-terbaru</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/03/23/Logo-BusinessWire-800x600.jpg</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Bolehkah beras merah dicampur beras putih? Ini penjelasannya</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:41:47 +0700</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Mencampur beras merah dan beras putih saat memasak nasi masih menjadi kebiasaan sebagian masyarakat yang ingin ...</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681840/bolehkah-beras-merah-dicampur-beras-putih-ini-penjelasannya</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/11/21/pexels-polina-tankilevitch-4110253.jpg</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DKI kemarin, rekayasa lalin terkait MRT hingga jumlah penduduk miskin</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:38:20 +0700</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Sejumlah berita seputar Jakarta pada Rabu (5/8) menarik untuk disimak kembali hari ini, mulai dari rekayasa lalu lintas ...</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681839/dki-kemarin-rekayasa-lalin-terkait-mrt-hingga-jumlah-penduduk-miskin</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/IMG_2392.jpeg</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Kenapa makan ubi bikin kentut? Ini penyebabnya menurut ahli gizi</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:33:01 +0700</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Makan ubi sering dikaitkan dengan meningkatnya frekuensi buang angin atau kentut. Anggapan tersebut ternyata memiliki ...</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681835/kenapa-makan-ubi-bikin-kentut-ini-penyebabnya-menurut-ahli-gizi</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/18/366068.jpg</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Vaksin HPV untuk siswa laki-laki</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:30:00 +0700</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan (Kemenkes) memperluas vaksinasi human papillomavirus (HPV) pada 2026 dengan menyasar siswa ...</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5681831/vaksin-hpv-untuk-siswa-laki-laki</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/20260806-Vaksin-HPV-untuk-siswa-laki-laki.jpg</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Sudah tidur 8 jam tapi masih lelah? Ini 8 tanda kualitas tidur buruk</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:27:38 +0700</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Banyak orang menganggap tidur selama tujuh hingga delapan jam sudah cukup untuk menjaga kesehatan. Padahal, durasi ...</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681829/sudah-tidur-8-jam-tapi-masih-lelah-ini-8-tanda-kualitas-tidur-buruk</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/03/tidur.jpg</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Sulit tidur? Coba 7 minuman alami yang bisa membantu cepat terlelap</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:22:00 +0700</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Tidur yang nyenyak menjadi salah satu kunci untuk menjaga kesehatan tubuh dan pikiran. Sayangnya, banyak orang masih ...</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681828/sulit-tidur-coba-7-minuman-alami-yang-bisa-membantu-cepat-terlelap</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2018/11/D1381D2E-B040-47E1-8DE3-1CD98B238FE5.jpeg</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Jipang Menyala, kreasi lampu hias semarakkan HUT ke-81 RI</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:20:11 +0700</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ANTARA - Warga Desa Jipang, Kecamatan Karanglewas, Kabupaten Banyumas, Jawa Tengah, memeriahkan HUT ke-81 Kemerdekaan ...</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5681791/jipang-menyala-kreasi-lampu-hias-semarakkan-hut-ke-81-ri</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/AYM_JIPANG-MENYALA-KREASI-LAMPU-HIAS.jpg</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Everton datangkan Christian Norgaard dari Arsenal</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:10:16 +0700</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Everton mendatangkan gelandang Christian Norgaard dari  Arsenal dalam skema transfer penuh dalam kontrak ...</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681824/everton-datangkan-christian-norgaard-dari-arsenal</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/f4176e00-910b-11f1-9e05-9b214625883c.jpg</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Sebagian Jakarta bakal cerah berawan pada Kamis pagi</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:06:32 +0700</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Badan Meteorologi Klimatologi dan Geofisika (BMKG) memprakirakan wilayah Jakarta Barat, Jakarta Pusat, Jakarta Selatan, ...</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681820/sebagian-jakarta-bakal-cerah-berawan-pada-kamis-pagi</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/19/IMG_20260719_000858.jpg</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Xsolla, GDAP, dan DTI-EMB Umumkan Kemitraan Strategis untuk Mempercepat Pertumbuhan Industri Game di Filipina</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:03:19 +0700</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>- Xsolla, sebuah perusahaan perdagangan game video global terkemuka, pada hari ini mengumumkan penandatanganan Nota ...</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681817/xsolla-gdap-dan-dti-emb-umumkan-kemitraan-strategis-untuk-mempercepat-pertumbuhan-industri-game-di-filipina</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Cara hilangkan bau sepatu yang membandel, ampuh dengan bahan sederhana</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 05:59:32 +0700</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Bau apek pada sepatu sering muncul akibat kelembapan, keringat, serta pertumbuhan bakteri dan jamur yang terperangkap ...</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681816/cara-hilangkan-bau-sepatu-yang-membandel-ampuh-dengan-bahan-sederhana</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/06/Festival-Sentra-Industri-Di-Bandung-060726-rai-3.jpg</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>BPS catat jumlah penduduk miskin di Sumsel turun 28 ribu orang</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 05:54:26 +0700</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Badan Pusat Statistik (BPS) mencatat jumlah penduduk miskin di Sumatera Selatan per Maret 2026 mencapai 869.970 orang ...</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681813/bps-catat-jumlah-penduduk-miskin-di-sumsel-turun-28-ribu-orang</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/a12529b8-8a2b-4d12-a36d-de767436b64d.jpeg</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>8 manfaat beras merah untuk kesehatan, bantu jaga gula darah</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:45:06 +0700</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Beras merah menjadi salah satu pilihan sumber karbohidrat yang semakin diminati masyarakat karena memiliki kandungan ...</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5681845/8-manfaat-beras-merah-untuk-kesehatan-bantu-jaga-gula-darah</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/20/pembukaan-jatiluwih-festival-2026-bali-200626-nhw-5.jpg</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bereskan Utang, Kemenkeu Ambil Alih 60% Saham Kereta Cepat September</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 06:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Kementerian Keuangan (Kemenkeu) mengambil seluruh saham PT Pilar Sinergi BUMN Indonesia (PSBI) di PT Kereta Cepat Indonesia China (KCIC).</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606067/bereskan-utang-kemenkeu-ambil-alih-60-saham-kereta-cepat-september</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/03/15/mobilitas-penumpang-whoosh-diprediksi-meningkat-saat-lebaran-1773573347987_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Pajak Toko Online Ditunda karena Ekonomi Belum Lari Kencang</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 05:55:00 +0700</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Kementerian Keuangan (Kemenkeu) menunda penerapan pajak e-commerce yang sebelumnya dijadwalkan mulai berlaku 1 Agustus 2026.</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606042/pajak-toko-online-ditunda-karena-ekonomi-belum-lari-kencang</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2019/01/14/ecf367f7-0e3e-4422-a3a4-1f35143e24a6_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I43"/>
+  <autoFilter ref="A1:I59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 06:43 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$257</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$330</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I257"/>
+  <dimension ref="A1:I330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12511,8 +12511,3439 @@
         </is>
       </c>
     </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Bapanas pastikan pasokan bawang putih aman dan terjaga</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:33:39 +0700</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Badan Pangan Nasional (Bapanas) memastikan pasokan bawang putih nasional tetap aman dan terjaga melalui penguatan ...</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682304/bapanas-pastikan-pasokan-bawang-putih-aman-dan-terjaga</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/FDA4BAED-1158-445D-9FD7-7209B487040C.jpeg</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Banggar DPR nilai faktor musiman dongkrak ekonomi RI tumbuh 5,2 persen</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:33:25 +0700</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Badan Anggaran Dewan Perwakilan Rakyat (Banggar DPR) RI menilai faktor musiman mendongkrak perekonomian RI tumbuh 5,2 ...</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682303/banggar-dpr-nilai-faktor-musiman-dongkrak-ekonomi-ri-tumbuh-52-persen</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/01/Said-Abdullah-1.jpg</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Personel Gulkarmat Jaksel padamkan kebakaran di SDN 04 Srengseng Sawah</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:32:38 +0700</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Sebanyak 60 personel Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Selatan (Jaksel) ...</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682300/personel-gulkarmat-jaksel-padamkan-kebakaran-di-sdn-04-srengseng-sawah</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001014476.jpg</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Hakim federal AS izinkan Trump akhiri perlindungan 350 warga Haiti</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:29:46 +0700</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Hakim federal Amerika Serikat (AS) berkedudukan di Washington D.C. mengabulkan keputusan pemerintahan Presiden Donald ...</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682297/hakim-federal-as-izinkan-trump-akhiri-perlindungan-350-warga-haiti</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000013_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>OnePlus meredup di pasar global, distribusi dihentikan di pasar AS</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:27:35 +0700</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Jenama ponsel pintar, OnePlus, tampak makin kehilangan eksistensinya di pasar global setelah baru-baru ini secara resmi ...</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682295/oneplus-meredup-di-pasar-global-distribusi-dihentikan-di-pasar-as</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/InShot_20260806_130451713.jpg</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Menaker dorong perkuat STEM guna hapus kesenjangan skill tenaga kerja</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:26:10 +0700</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli mendorong penguatan pendidikan Sains, Teknologi, Rekayasa, dan Matematika ...</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682292/menaker-dorong-perkuat-stem-guna-hapus-kesenjangan-skill-tenaga-kerja</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000470811.jpg</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Komisi IX ingatkan nakes jaga etika bermedia sosial</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:24:33 +0700</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Anggota Komisi IX DPR RI Asep Rommy Romaya mengingatkan tenaga kesehatan (nakes) untuk menjaga etika dalam bermedia ...</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682289/komisi-ix-ingatkan-nakes-jaga-etika-bermedia-sosial</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/09/WhatsApp-Image-2026-06-09-at-14.50.10.jpeg</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>BI: Transaksi QRIS capai 12,55 miliar pada semester I 2026</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:23:46 +0700</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Bank Indonesia (BI) mencatat volume transaksi digital Quick Response Code Indonesian Standard atau QRIS menembus 12,55 ...</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682285/bi-transaksi-qris-capai-1255-miliar-pada-semester-i-2026</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_20260806_134312.jpg</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Lima alutsista baru TNI AU dikerahkan dalam latihan gabungan TNI</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:20:48 +0700</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Lima alat utama sistem senjata (alutsista) milik TNI AU diturunkan untuk mengikuti latihan gabungan TNI terintegrasi ...</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682283/lima-alutsista-baru-tni-au-dikerahkan-dalam-latihan-gabungan-tni</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001560157.jpg</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Potret peluncuran Satelit Lampung-1 di Shandong</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:20:41 +0700</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Roket pengangkut Jielong-3 Y12 lepas landas dari perairan lepas pantai Kota Haiyang, Provinsi Shandong, China timur, ...</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682279/potret-peluncuran-satelit-lampung-1-di-shandong</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000033_20260805_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>BPS rilis Indeks Kepuasan Layanan Haji Indonesia 2026 capai 83,28 poin</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:18:15 +0700</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Badan Pusat Statistik (BPS) merilis hasil Indeks Kepuasan Layanan Haji Indonesia (IKLHI) tahun 1447 Hijriah/2026 Masehi ...</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682276/bps-rilis-indeks-kepuasan-layanan-haji-indonesia-2026-capai-8328-poin</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000176812.jpg</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Penggunaan Air KAI Turun 22,16 Persen, ATWP LRT Jabodebek Perkuat Daur Ulang Air</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:15:37 +0700</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) mencatat penggunaan air sebesar 716,30 megaliter sepanjang 2025. Jumlah tersebut ...</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682272/penggunaan-air-kai-turun-2216-persen-atwp-lrt-jabodebek-perkuat-daur-ulang-air</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-12.19.53.jpeg</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Ekspedisi Rupiah Berdaulat 2026 sambangi Papua</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:15:00 +0700</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Ekspedisi Rupiah Berdaulat (ERB) menjangkau Papua pada 4-10 Agustus 2026 untuk memastikan masyarakat di wilayah ...</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/infografik/5682263/ekspedisi-rupiah-berdaulat-2026-sambangi-papua</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/20260806-Ekspedisi-Rupiah-Berdaulat-2026-sambangi-Papua.jpg</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>BRIN paparkan 12 klaster inovasi kepada Presiden Prabowo</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:14:49 +0700</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Sebanyak 150 peneliti Badan Riset dan Inovasi Nasional (BRIN) memaparkan hasil riset dan inovasi dalam 12 klaster ...</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682268/brin-paparkan-12-klaster-inovasi-kepada-presiden-prabowo</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000034735.jpg</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Polisi dalami dugaan hubungan sesama jenis dalam kasus mutilasi di Depok</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:09:26 +0700</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Polda Metro Jaya mendalami dugaan adanya hubungan sesama jenis antara tersangka SA alias Saepullah dengan korban dalam ...</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682267/polisi-dalami-dugaan-hubungan-sesama-jenis-dalam-kasus-mutilasi-di-depok</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/IMG_4065.jpeg</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Anthropic bentuk tim pengembangan chip untuk AI Claude</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:04:28 +0700</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Perusahaan kecerdasan artifisial (AI) Anthropic membentuk tim khusus untuk mengembangkan chip AI buatan sendiri untuk ...</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682260/anthropic-bentuk-tim-pengembangan-chip-untuk-ai-claude</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/06/InShot_20260506_133536251.jpg</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>210,47 Juta Pelanggan Commuter Line Jabodetabek Perkuat Produktivitas dan Mobilitas Rendah Karbon</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:01:55 +0700</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) melayani 210.468.029 pelanggan Commuter Line Jabodetabek sepanjang ...</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682256/21047-juta-pelanggan-commuter-line-jabodetabek-perkuat-produktivitas-dan-mobilitas-rendah-karbon</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-12.09.05.jpg</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Mendukbangga minta SPPG aktif salurkan MBG 3B di Babel</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:01:20 +0700</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>ANTARA - Menteri Kependudukan dan Pembangunan Keluarga (Mendukbangga) / Kepala Badan Kependudukan dan Keluarga ...</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5682220/mendukbangga-minta-sppg-aktif-salurkan-mbg-3b-di-babel</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/MENDUKBANGGA-MINTA-SPPG-AKTIF-SALURKAN-MBG-3B-DI-BABEL.jpg</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Sekolah Rakyat Medan: Membangun karakter demi masa depan siswa</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:00:59 +0700</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Para siswa dari berbagai jenjang pendidikan tampak menyimak materi dalam program Taruna Mengajar di Sekolah Rakyat ...</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682255/sekolah-rakyat-medan-membangun-karakter-demi-masa-depan-siswa</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG-20260806-WA0034-2.jpg</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>KPK panggil anggota DPRD Kaltim di kasus Rita Widyasari</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:00:12 +0700</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi (KPK) memanggil anggota DPRD Kalimantan Timur Sarkowi V. Zahry sebagai saksi dalam ...</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682253/kpk-panggil-anggota-dprd-kaltim-di-kasus-rita-widyasari</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_7484.jpg</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Dishub DKI uji coba penutupan perputaran arah di RS Fatmawati Raya</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:57:01 +0700</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Dinas Perhubungan (Dishub) DKI Jakarta melakukan uji coba penutupan perputaran arah (U-turn) di Jalan RS Fatmawati ...</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682252/dishub-dki-uji-coba-penutupan-perputaran-arah-di-rs-fatmawati-raya</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001014312.jpg</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>PAN: Usulan Pilkada tanpa wakil sudah jadi diskusi lintas fraksi</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:55:59 +0700</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Wakil Ketua Umum Partai Amanat Nasional (PAN) Saleh Partaonan Daulay menilai usulan pemilihan kepala daerah (Pilkada) ...</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682251/pan-usulan-pilkada-tanpa-wakil-sudah-jadi-diskusi-lintas-fraksi</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/24/1001249216.jpg</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Sergio Castel ungkap target bersama Persik Kediri</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:55:46 +0700</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Penyerang anyar Sergio Castel mengungkapkan targetnya telah menerima tawaran bergabung bersama klub BRI Super League ...</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682247/sergio-castel-ungkap-target-bersama-persik-kediri</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/10/persib-bandung-kalahkan-persija-jakarta-2787353.jpg</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Kuasa hukum: Praperadilan Febrie bukan hindari proses hukum</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:54:32 +0700</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Tim kuasa hukum mantan Jaksa Agung Muda Tindak Pidana Khusus (Jampidsus) Febrie Adriansyah menyatakan permohonan ...</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682243/kuasa-hukum-praperadilan-febrie-bukan-hindari-proses-hukum</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/febrie-adriansyah-ajukan-praperadilan-ke-pn-jaksel-2835015.jpg</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>SpaceX berencana buat Starlink jadi opsel di AS</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:51:06 +0700</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Perusahaan antariksa yang dimiliki pebisnis Elon Musk, SpaceX, membagikan rencana barunya untuk masuk ke dalam industri ...</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682241/spacex-berencana-buat-starlink-jadi-opsel-di-as</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/01/09/IMG-20241208-WA0015_1.jpg</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Gulkarmat Jaktim evakuasi musang yang jatuh dari plafon rumah warga</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:50:38 +0700</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Petugas Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Timur (Jaktim) mengevakuasi seekor ...</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682240/gulkarmat-jaktim-evakuasi-musang-yang-jatuh-dari-plafon-rumah-warga</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/InShot_20260806_115833896.jpg</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Komisioner Uni Eropa: Penyelundup bertanggung jawab atas tragedi Ceuta</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:46:44 +0700</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Komisioner Uni Eropa (EU) untuk Urusan Dalam Negeri dan Migrasi Magnus Brunner meyakini bahwa penyelundup manusia ...</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682237/komisioner-uni-eropa-penyelundup-bertanggung-jawab-atas-tragedi-ceuta</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Spanyol-Migran-memasuki-Ceuta.jpg</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Bandara utama Venezuela kembali Layani penerbangan kargo pascagempa</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:45:28 +0700</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Bandar Udara (Bandara) Internasional Simon Bolivar, bandara utama yang melayani ibu kota Venezuela, Caracas, kembali ...</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682235/bandara-utama-venezuela-kembali-layani-penerbangan-kargo-pascagempa</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000009_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>128.331 warga daftar undangan upacara HUT Ke-81 RI di Istana</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:45:26 +0700</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Sebanyak 128.331 pendaftar dari 36 provinsi di Indonesia dan 14 negara mengikuti pendaftaran undangan Upacara ...</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682231/128331-warga-daftar-undangan-upacara-hut-ke-81-ri-di-istana</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/prasetyo-hadi_1.jpeg</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>KAI Layani 1,57 Juta Ton Angkutan BBM hingga Juli 2026, Jaga Kelancaran Rantai Pasok Energi Nasional</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:43:01 +0700</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>PT Kereta Api Indonesia (Persero) melayani angkutan bahan bakar minyak atau BBM sebanyak 1.570.911 ton selama ...</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682227/kai-layani-157-juta-ton-angkutan-bbm-hingga-juli-2026-jaga-kelancaran-rantai-pasok-energi-nasional</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-12.05.34.jpeg</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Kapolda-Pangdam perkuat sinergi lewat kunjungan ke Mako Brimob</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:41:50 +0700</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya Komjen Pol. Asep Edi Suheri bersama Pangdam Jaya Letjen TNI Deddy Suryadi memperkuat sinergi ...</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682225/kapolda-pangdam-perkuat-sinergi-lewat-kunjungan-ke-mako-brimob</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Polda-Pangdam.jpg</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>PSS Sleman gelar peluncuran tim di Stadion Maguwoharjo</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:40:06 +0700</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Klub Promosi BRI Super League PSS Sleman akan menggelar peluncuran tim untuk menghadapi kompetisi 2026/2027 di Stadion ...</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682221/pss-sleman-gelar-peluncuran-tim-di-stadion-maguwoharjo</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2021/04/23/IMG_5232-scaled-e1619170570649-1024x745.jpg</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Minecraft akan dirilis untuk Nintendo Switch 2 pada 27 Oktober</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:37:53 +0700</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>Gim Minecraft akan hadir di konsol Nintendo Switch 2 pada 27 Oktober 2026 dengan peningkatan kualitas visual ...</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682219/minecraft-akan-dirilis-untuk-nintendo-switch-2-pada-27-oktober</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Homepage_Discover-our-games_MC-Vanilla-KeyArt_864x864.jpg</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Kepala Bapanas pastikan pengawasan beras fortifikasi diperketat</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:32:09 +0700</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Kepala Badan Pangan Nasional (Bapanas) sekaligus Menteri Pertanian Andi Amran Sulaiman memastikan pengawasan beras ...</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682216/kepala-bapanas-pastikan-pengawasan-beras-fortifikasi-diperketat</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/8813B57A-20AF-421A-B253-891224E6867C.jpeg</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>6 investasi TPT ciptakan hampir 10 ribu lapangan kerja</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:29:38 +0700</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Sekretaris Jenderal Asosiasi Garment dan Textile Indonesia (AGTI) Rizal Tanzil Rakhman mengatakan investasi pada enam ...</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682213/6-investasi-tpt-ciptakan-hampir-10-ribu-lapangan-kerja</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/14/antarafoto-kinerja-industri-manufaktur-tahun-2024-150124-ysw-2.jpg</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Wamenpar dorong investasi industri rekreasi lewat Fun Asia Expo 2026</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:28:47 +0700</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Pariwisata Ni Luh Puspa mengatakan penyelenggaraan Fun Asia Expo 2026 menjadi upaya untuk mendorong ...</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682211/wamenpar-dorong-investasi-industri-rekreasi-lewat-fun-asia-expo-2026</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-05-at-21.41.39.jpeg</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Hiroshima serukan hapus senjata nuklir pada peringatan 81 thn bom atom</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:27:55 +0700</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Hiroshima pada Kamis menyerukan penghapusan senjata nuklir oleh para pemimpin dunia di tengah meningkatnya ...</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682207/hiroshima-serukan-hapus-senjata-nuklir-pada-peringatan-81-thn-bom-atom</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/ilustrasi-peringatan-bom-atom-Jepang.jpg</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Koalisi Pejalan Kaki minta JPO kawasan UI hingga Pasar Minggu direnovasi</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:27:20 +0700</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Koalisi Pejalan Kaki meminta pemerintah agar merenovasi jembatan penyeberangan orang (JPO) Stasiun Universitas ...</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682205/koalisi-pejalan-kaki-minta-jpo-kawasan-ui-hingga-pasar-minggu-direnovasi</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001014293.jpg</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>OJK minta pindar perkuat tata kelola demi jaga kepercayaan publik</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:22:41 +0700</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Otoritas Jasa Keuangan (OJK) meminta industri pinjaman daring (pindar) memperkuat tata kelola dan manajemen risiko guna ...</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682203/ojk-minta-pindar-perkuat-tata-kelola-demi-jaga-kepercayaan-publik</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/c756d23e-0e38-4da7-a296-05d8e08704f4.jpeg</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>PWI nilai pers punya peran strategis untuk memerangi pinjol ilegal</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:22:28 +0700</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Ketua Umum Persatuan Wartawan Indonesia (PWI) Pusat Akhmad Munir menilai pers memiliki peran strategis dalam ...</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682199/pwi-nilai-pers-punya-peran-strategis-untuk-memerangi-pinjol-ilegal</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/f54d1eff-1fa0-484e-aa29-cf7df6459230.jpeg</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Huawei Nova 16 SE meluncur dengan layar OLED dan baterai 8.500 mAh</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:20:30 +0700</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Huawei resmi menghidupkan kembali lini ponsel Nova SE setelah absen lebih dari dua tahun dengan meluncurkan Huawei Nova ...</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682197/huawei-nova-16-se-meluncur-dengan-layar-oled-dan-baterai-8500-mah</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Huawei-Nova-16-SE.jpg</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Tinjau SPPG Pangkalpinang, Mendukbangga pastikan kualitas MBG 3B</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:18:57 +0700</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Menteri Kependudukan dan Pembangunan Keluarga (Mendukbangga) Wihaji meninjau Satuan Pelayanan Pemenuhan Gizi (SPPG) di ...</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682195/tinjau-sppg-pangkalpinang-mendukbangga-pastikan-kualitas-mbg-3b</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/mendukbangga.jpg</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Waktu terbaik naik pesawat bersama anak agar nyaman dan minim jet lag</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:16:37 +0700</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Waktu keberangkatan pesawat dapat memengaruhi kenyamanan anak selama perjalanan sekaligus membantu mengurangi risiko ...</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682193/waktu-terbaik-naik-pesawat-bersama-anak-agar-nyaman-dan-minim-jet-lag</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2013/09/20130902pengasuh-anak-dalam-pesawat.jpg</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Menteri PPN buka Indonesia's Sustainable Development Goals Award 2026</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:15:22 +0700</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Menteri Perencanaan Pembangunan Nasional/Kepala Badan Perencanaan Pembangunan Nasional (PPN/Bappenas) Rachmat Pambudy ...</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682191/menteri-ppn-buka-indonesias-sustainable-development-goals-award-2026</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/PPN-Judol.jpeg</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Operasi kereta Daop 2 kemabli normal pascagempa walau telat 9-60 menit</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:15:20 +0700</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>PT KAI Daerah Operasi (Daop) 2 Bandung mengungkapkan perjalanan kereta api telah kembali beroperasi normal ...</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682187/operasi-kereta-daop-2-kemabli-normal-pascagempa-walau-telat-9-60-menit</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1002080940.jpg</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>KPK panggil Rudy Tanoe sebagai saksi kasus penyaluran bansos beras</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:14:06 +0700</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi (KPK) memanggil Komisaris Utama PT Dosni Roha Logistik sekaligus Direktur Utama PT Dosni ...</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682185/kpk-panggil-rudy-tanoe-sebagai-saksi-kasus-penyaluran-bansos-beras</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/12/14/Screenshot_20231214_140224_Video-Player.jpg</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Kemendikdasmen telusuri dugaan penyalahgunaan Dapodik murid</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:12:19 +0700</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Kementerian Pendidikan Dasar dan Menengah (Kemendikdasmen) tengah melakukan verifikasi dan penelusuran terhadap dugaan ...</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682181/kemendikdasmen-telusuri-dugaan-penyalahgunaan-dapodik-murid</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/06/25/pendidikan.jpg</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>KSOP Sampit keluarkan maklumat pelayaran waspada kabut asap karhutla</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:12:14 +0700</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Kantor Kesyahbandaran dan Otoritas Pelabuhan (KSOP) Kelas III Sampit, Kabupaten Kotawaringin Timur (Kotim), Kalimantan ...</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682180/ksop-sampit-keluarkan-maklumat-pelayaran-waspada-kabut-asap-karhutla</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001725985.jpg</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Indonesia tekankan kepatuhan pada hukum laut dalam konflik bersenjata</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:10:27 +0700</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Indonesia mendorong kepatuhan terhadap hukum lingkungan laut serta menyoroti perlunya pedoman teknis mengenai perlakuan ...</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682176/indonesia-tekankan-kepatuhan-pada-hukum-laut-dalam-konflik-bersenjata</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Kemlu-RI-Naval-Warfare-Workstream-ICRC-06082026_1.jpg</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Membangun Masa Depan Riset dan Teknologi, Pembangunan Gedung L-SSIT Universitas Udayana Capai Progres 47,11%</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:10:21 +0700</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Pembangunan Gedung Laboratorium Smart System and Integrated Technologies (L-SSIT) Universitas Udayana, Bali terus ...</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682175/membangun-masa-depan-riset-dan-teknologi-pembangunan-gedung-l-ssit-universitas-udayana-capai-progres-4711</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Pembangunan-Gedung-L-SSIT.jpg</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>OJK didorong siapkan mitigasi risiko kredit macet industri pindar</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:05:25 +0700</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Konsultan dan Perencana Keuangan Elvi Diana mendorong Otoritas Jasa Keuangan (OJK) menyiapkan langkah mitigasi terhadap ...</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682173/ojk-didorong-siapkan-mitigasi-risiko-kredit-macet-industri-pindar</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/30/IMG_0468.jpeg</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Cinta Indonesia, Dubes Palestina Akan Gelar Perayaan HUT RI di Kedubes</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:32:50 +0700</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Duta Besar Palestina, Al-Sattiri, mengumumkan perayaan HUT ke-79 RI sebagai ungkapan terima kasih rakyat Palestina. Gubernur DKI Jakarta mendukung acara ini.</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606839/cinta-indonesia-dubes-palestina-akan-gelar-perayaan-hut-ri-di-kedubes</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/pramono-bersama-dubes-palestina-brigitta-belia-permata-saridetikcom-1785997942304_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>150 Peneliti BRIN Bakal Paparkan Hasil Riset Pangan hingga Nuklir ke Prabowo</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:32:06 +0700</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Kepala Badan Riset dan Inovasi Nasional (BRIN) Arif Satria membawa 150 orang peneliti ke Istana, Jakarta.</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606837/150-peneliti-brin-bakal-paparkan-hasil-riset-pangan-hingga-nuklir-ke-prabowo</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kepala-brin-arif-satria-evadetikcom-1785997911603_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Presiden Iran Ungkap Komunikasi dengan Mojtaba Khamenei 'Sangat Sulit'</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:27:08 +0700</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Novi Christiastuti</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Presiden Iran Masoud Pezeshkian mengungkapkan bahwa komunikasi dengan pemimpin tertinggi negaranya, Mojtaba Khamenei, sangat sulit pada saat ini.</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606829/presiden-iran-ungkap-komunikasi-dengan-mojtaba-khamenei-sangat-sulit</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/11/pemimpin-tertinggi-iran-mojtaba-khamenei-1775906157579_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Bamsoet Ingatkan Industri Kesehatan Harus Adaptif Hadapi Tantangan Global</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:18:43 +0700</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Bamsoet soroti tantangan industri rumah sakit di tengah ketidakpastian ekonomi. Siloam Hospitals menunjukkan pertumbuhan positif dan inovasi layanan kesehatan.</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606810/bamsoet-ingatkan-industri-kesehatan-harus-adaptif-hadapi-tantangan-global</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/bamsoet-1785997067503_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Istri di Bogor Bakar Baju Suami hingga Rumah Terbakar, Dipicu Cekcok</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:07:22 +0700</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Muchamad Sholihin</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Kebakaran rumah di Menteng Asri, Bogor, dipicu istri yang membakar baju suami saat bertengkar. Kerugian mencapai Rp 150 juta.</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606787/istri-di-bogor-bakar-baju-suami-hingga-rumah-terbakar-dipicu-cekcok</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kebakaran-rumah-di-bogor-dipicu-istri-bakar-baju-suami-1785996380774_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Pengedar Ribuan Tramadol dan Hexymer Dibekuk di Tangerang, Pemasok Diburu</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:52:13 +0700</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Polres Metro Tangerang Kota mengungkap peredaran obat keras ilegal, menangkap tersangka YG dengan ribuan butir tramadol dan hexymer.</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606762/pengedar-ribuan-tramadol-dan-hexymer-dibekuk-di-tangerang-pemasok-diburu</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2023/07/25/ilustrasi-penangkapan_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Kobra di Karanganyar Telan Pisau hingga Perut Terbelah, Diduga Stres</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:48:58 +0700</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Agil Trisetiawan Putra</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Seekor ular kobra ditemukan dalam kondisi menelan pisau dapur di rumah warga Desa Sroyo, Kecamatan Jaten, Kabupaten Karanganyar.</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606756/kobra-di-karanganyar-telan-pisau-hingga-perut-terbelah-diduga-stres</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/ular-kobra-menelan-pisau-di-desa-sroyo-jaten-karanganyar-tanpa-watermark-1785911516116_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Polres Serang Kirim 64 Truk Tangki Air Atasi Kekeringan di 6 Kecamatan</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:48:44 +0700</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Polres Serang mengirim 64 tangki air untuk membantu warga di daerah terdampak kekeringan.</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606754/polres-serang-kirim-64-truk-tangki-air-atasi-kekeringan-di-6-kecamatan</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/polres-serang-mengirim-64-tangki-air-untuk-membantu-warga-di-daerah-terdampak-kekeringan-1785995228316_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Buron Kasus Pembunuhan Sekdin PRKP Bangkalan Diduga Gondol Emas 1 Kg</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:44:25 +0700</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Suparno</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Buron kasus kematian Sekdin PRKP Bangkalan, Erlan, diduga mencuri perhiasan emas 1 kg dan uang tunai ratusan juta. Keluarga korban melaporkan kehilangan.</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606748/buron-kasus-pembunuhan-sekdin-prkp-bangkalan-diduga-gondol-emas-1-kg</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/07/pembunuhan-sekdin-prkp-bangkalan-1783403824762_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Netanyahu Tegaskan Tolak Kesepakatan Gaza Usulan Trump</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:43:46 +0700</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Novi Christiastuti</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Netanyahu menegaskan penolakannya terhadap kesepakatan perdamaian Gaza yang diusulkan sekutu dekatnya, Presiden AS Donald Trump.</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606747/netanyahu-tegaskan-tolak-kesepakatan-gaza-usulan-trump</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/26/pm-israel-benjamin-netanyahu-1756180921129_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Perkuat Sinergi TNI-Polri, Kapolda Metro dan Pangdam Jaya Kunjungi Dankorbrimob Polri</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:33:56 +0700</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Kapolda Metro Jaya dan Pangdam Jaya kunjungi Markas Korps Brimob untuk memperkuat sinergi TNI-Polri dalam menjaga keamanan Jakarta dan dukung agenda nasional.</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606739/perkuat-sinergi-tni-polri-kapolda-metro-dan-pangdam-jaya-kunjungi-dankorbrimob-polri</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kapolda-metro-jaya-dan-pangdam-jaya-mengunjungi-dankorbrimob-polri-dalam-rangka-memperkuat-soliditas-dan-sinergi-tni-polri-1785994408613_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>SDN di Srengseng Jaksel Kebakaran: Pelajar Dievakuasi, Api Berangsur Mati</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:28:19 +0700</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Bangunan SDN di Srengseng Sawah, Jagakarsa, Jakarta Selatan, dilanda kebakaran. Pelajar di sekolah tersebut sudah dievakuasi.</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606722/sdn-di-srengseng-jaksel-kebakaran-pelajar-dievakuasi-api-berangsur-mati</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/01/07/1ec4fbfe-119d-4c1c-b3e0-e50685a1e1bb_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>PK Ditolak, Bos Smelter Tetap Dihukum 18 Tahun Bui di Kasus Korupsi Rp 300 T</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:26:41 +0700</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Mahkamah Agung (MA) menolak peninjauan kembali (PK) yang diajukan terpidana kasus korupsi pengelolaan timah bernama Tamron.</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606719/pk-ditolak-bos-smelter-tetap-dihukum-18-tahun-bui-di-kasus-korupsi-rp-300-t</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/01/26/aed271bd-0523-49d3-a57f-ee5dd7541d42_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>SD di Cibaduyut Digembok Ahli Waris, Hampir Seribu Siswa Terpaksa Pulang</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:20:57 +0700</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Rifat Alhamidi</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Sebanyak 945 siswa SDN 026 Bojongloa, Kota Bandung, tak bisa belajar seperti biasa. Pasalnya, lingkungan sekolah itu disegel oleh ahli waris.</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606702/sd-di-cibaduyut-digembok-ahli-waris-hampir-seribu-siswa-terpaksa-pulang</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/pembelajaran-sdn-026-bojongloa-dihentikan-setelah-sempat-disegel-ahli-waris-1785991246958_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Legislator PKB Usul Pilkada Tanpa Wakil, PAN: Usulan Bagus dan Simpatik</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:07:39 +0700</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Usulan ini bagus dan simpatik. Sudah banyak diperbincangkan di lintas fraksi, kata Saleh.</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606676/legislator-pkb-usul-pilkada-tanpa-wakil-pan-usulan-bagus-dan-simpatik</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/05/10/saleh-daulay_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>SDN di Srengseng Sawah Jaksel Kebakaran</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:04:32 +0700</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Bangunan sekolah dasar negeri (SDN) di Srengseng Sawah, Jagakarsa, Jaksel dilanda kebakaran. Petugas damkar berjibaku memadamkan api.</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606674/sdn-di-srengseng-sawah-jaksel-kebakaran</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2015/11/23/aba98b4b-9134-44d4-bc2c-056cf42d0c43_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Kenalkan, Sofia Anak Buruh Lulusan SMA CT ARSA yang Tembus ITB</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:01:15 +0700</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Nur Khansa Ranawati</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Bagi Sofi Aulia Syarifa (19), melanjutkan pendidikan hingga kuliah pernah terasa seperti mimpi. Kini, SMA Plus CT ARSA Sukoharjo itu resmi jadi mahasiswa ITB.</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606666/kenalkan-sofia-anak-buruh-lulusan-sma-ct-arsa-yang-tembus-itb</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/sofi-aulia-syarifa-lulusan-sma-plus-ct-arsa-yang-tembus-itb-1785923838256_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Penyu Hendak Bertelur Mati Terbelah di Kaltim, Seluruh Telurnya Diambil Pelaku</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 11:31:33 +0700</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Riani Rahayu</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>Seekor penyu betina yang hendak bertelur mati terbelah di pesisir Kabupaten Berau, Kaltim. Seluruh telur yang masih ada di dalam tubuh penyu itu hilang.</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606620/penyu-hendak-bertelur-mati-terbelah-di-kaltim-seluruh-telurnya-diambil-pelaku</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/penyu-ditemukan-mati-mengenaskan-di-pesisir-berau-1785936713273_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Roy Suryo Kalah Lagi di Praperadilan Ketiga</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 10:34:01 +0700</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Rumondang Naibaho</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Hakim Pengadilan Negeri Jakarta Selatan tak menerima gugatan praperadilan ketiga yang diajukan oleh Roy Suryo.</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606515/roy-suryo-kalah-lagi-di-praperadilan-ketiga</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/sidang-praperadilan-roy-suryo-rumondangdetikcom-1785987232013_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Kemenhan Rotasi 14 Pejabat Tinggi, Sekretaris Bacadnas Berganti</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:43:27 +0700</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Kemenhan merotasi 14 pejabat pimpinan tinggi, termasuk posisi Sekretaris Bacadnas yang kini dijabat Mayjen TNI (Mar) Freddy Ardianzah.</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/06/13424791/kemenhan-rotasi-14-pejabat-tinggi-sekretaris-bacadnas-berganti</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/1tcSy0VFMv_5jsqfG3Us-zZzC4I=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a742928e8f6f.jpg</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Terungkap Motif Penebangan 10 Pohon di Cihapit, Diduga demi Sewa Videotron</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:43:30 +0700</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Petinggi subkontraktor diduga memerintahkan penebangan 10 pohon di Cihapit karena berencana menyewa videotron yang pandangannya terhalang.</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/08/06/133000978/terungkap-motif-penebangan-10-pohon-di-cihapit-diduga-demi-sewa-videotron</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/u_bm11Ybowq4LB5HrbaMY629JB8=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a72e08497f56.jpg</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Satelit Lampung-1 Sukses Mengorbit, Mengapa Pemprov Belum Bisa Langsung Manfaatkan Datanya?</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:43:31 +0700</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Meski telah sukses diluncurkan ke orbit, data Satelit Lampung-1 masih harus melalui proses verifikasi dan pengolahan bersama BRIN sebelum digunakan.</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/06/131123978/satelit-lampung-1-sukses-mengorbit-mengapa-pemprov-belum-bisa-langsung</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/lt-GVFMNLaiVoB0qgnwsx5KS_Uw=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a741c7c0f5ae.jpg</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I257"/>
+  <autoFilter ref="A1:I330"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 07:14 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$330</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$376</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I330"/>
+  <dimension ref="A1:I376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -15942,8 +15942,2170 @@
         </is>
       </c>
     </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Beijing ditetapkan sebagai ibu kota arsitektur dunia UNESCO-UIA 2029</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:01:16 +0700</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Beijing ditetapkan sebagai Ibu Kota Arsitektur Dunia UNESCO-UIA (International Union of Architects) 2029, demikian ...</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682343/beijing-ditetapkan-sebagai-ibu-kota-arsitektur-dunia-unesco-uia-2029</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000012_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>AS cabut sanksi maskapai Irak, bantah longgarkan sanksi Iran</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:59:47 +0700</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>Departemen Keuangan Amerika Serikat (AS) mencabut sanksi untuk maskapai penerbangan asal Irak, Fly Baghdad, beserta dua ...</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682341/as-cabut-sanksi-maskapai-irak-bantah-longgarkan-sanksi-iran</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000008_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Pemprov DKI perkuat pendidikan anak sejak usia dini</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:58:33 +0700</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta terus berupaya memperkuat pendidikan sejak usia dini sebagai bagian dari ...</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682340/pemprov-dki-perkuat-pendidikan-anak-sejak-usia-dini</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000315491.jpg</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Menko Airlangga: Investasi sudah lebih merata di semester I 2026</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:56:01 +0700</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator (Menko) Bidang Perekonomian Airlangga Hartarto mengatakan kegiatan investasi sudah menunjukkan ...</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682336/menko-airlangga-investasi-sudah-lebih-merata-di-semester-i-2026</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_0438.jpeg</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Dishub Cilegon tertibkan parkir liar kendaraan di JLS</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:52:47 +0700</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>ANTARA - Dinas Perhubungan Kota Cilegon bersama Satlantas Polres Cilegon, Kamis (6/8), melaksanakan penertiban parkir ...</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5682307/dishub-cilegon-tertibkan-parkir-liar-kendaraan-di-jls</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/DISHUB-CILEGON-TERTIBKAN-PARKIR-LIAR-KENDARAAN-DI-JLS.jpg</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>BPS rilis IKLHI 2026, Menhaj: Alhamdulillah, pelayanan haji luar biasa</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:51:26 +0700</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Menteri Haji dan Umrah (Menhaj) Mochammad Irfan Yusuf menyebut capaian Indeks Kepuasan Layanan Haji Indonesia ...</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682333/bps-rilis-iklhi-2026-menhaj-alhamdulillah-pelayanan-haji-luar-biasa</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000176834.jpg</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>TNI AU pertajam kemampuan personel di bidang intelijen</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:47:34 +0700</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>TNI AU berupaya memperkuat kemampuan personelnya dalam bidang intelijen dengan menggelar Pelatihan Kepala Satuan ...</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682332/tni-au-pertajam-kemampuan-personel-di-bidang-intelijen</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001560248.jpg</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>"Desa Batu" di China Utara pikat wisatawan saat liburan musim panas</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:46:24 +0700</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Dikenal sebagai "desa batu", Desa Xijingyu di Distrik Jizhou, Kota Tianjin, China utara, terkenal dengan ...</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682328/desa-batu-di-china-utara-pikat-wisatawan-saat-liburan-musim-panas</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000005_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Sidang putusan praperadilan ketiga Roy Suryo</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:46:04 +0700</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Hakim tunggal I Ketut Darpawan memimpin jalannya sidang putusan praperadilan ketiga yang diajukan oleh tersangka kasus ...</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5682324/sidang-putusan-praperadilan-ketiga-roy-suryo</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Sidang-putusan-praperadilan-ketiga-Roy-Suryo-06082026-ab-1.jpg</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Wisatawan mancanegara menjajal pencapaian iptek China di Shenzhen</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:43:03 +0700</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Seiring penerapan mendalam dari pencapaian industri-industri emerging, banyak wisatawan mancanegara memilih wisata ilmu ...</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682320/wisatawan-mancanegara-menjajal-pencapaian-iptek-china-di-shenzhen</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000007_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Myanmar lestarikan 6.105 bangunan berusia seabad lebih</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:43:02 +0700</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>Pemerintah Myanmar melestarikan 6.105 bangunan yang berusia lebih dari 100 tahun dengan menetapkannya sebagai cagar ...</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682317/myanmar-lestarikan-6105-bangunan-berusia-seabad-lebih</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000010_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Pemprov DKI tegaskan dukung hak rakyat Palestina</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:42:21 +0700</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) DKI Jakarta menegaskan sikap mendukung hak rakyat Palestina untuk hidup dalam perdamaian, ...</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682315/pemprov-dki-tegaskan-dukung-hak-rakyat-palestina</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_2404.jpeg</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Menko IPK minta konsolidasi BUMN bisa dukung kawasan industri</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:40:18 +0700</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Infrastruktur dan Pembangunan Kewilayahan (Menko IPK) Agus Harimurti Yudhoyono (AHY) meminta ...</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682312/menko-ipk-minta-konsolidasi-bumn-bisa-dukung-kawasan-industri</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_5281.jpeg</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>BRIN pamerkan 150–200 produk inovasi kepada Presiden</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:39:30 +0700</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>Badan Riset dan Inovasi Nasional (BRIN) memamerkan sekitar 150–200 produk inovasi dari 12 klaster riset kepada ...</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682311/brin-pamerkan-150-200-produk-inovasi-kepada-presiden</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000034738.jpg</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>POSSI: Kejuaraan Asia 2026 jadi momentum populerkan hoki bawah air</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:39:02 +0700</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Pengurus Besar Persatuan Olahraga Selam Seluruh Indonesia (PB POSSI) menjadikan Kejuaraan Asia Hoki Bawah Air CMAS 2026 ...</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682309/possi-kejuaraan-asia-2026-jadi-momentum-populerkan-hoki-bawah-air</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/11/16/WhatsApp-Image-2025-11-15-at-18.51.38.jpeg</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Mendukbangga manfatkan ruang ramah anak, tekan gangguan mental remaja</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:35:34 +0700</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Menteri Kependudukan dan Pembangunan Keluarga (Mendukbangga) Wihaji mengintensifkan ruang ramah anak guna menjaga ...</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682308/mendukbangga-manfatkan-ruang-ramah-anak-tekan-gangguan-mental-remaja</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/mendukbangga2.jpg</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Kobra Telan Pisau di Karanganyar karena Stres? Ini Penjelasan Pakar UGM</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:05:41 +0700</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Tim detikJateng</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Pakar satwa UGM mengatakan ular memang bisa stres pada kondisi tertentu. Namun pada kasus ular kobra menelan pisau di Karanganyar, pakar punya pandangan lain.</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606905/kobra-telan-pisau-di-karanganyar-karena-stres-ini-penjelasan-pakar-ugm</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/ular-kobra-menelan-pisau-di-desa-sroyo-jaten-karanganyar-tanpa-watermark-1785911516116_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>BRIN Bawa Sepatu Buatan Sendiri Saat Temui Prabowo, Mau Diproduksi Massal</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:04:30 +0700</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Kepala Badan Riset dan Inovasi Nasional (BRIN) Arif Satria memamerkan sepatu buatan lembaganya saat hendak menemui Presiden Prabowo Subianto.</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606902/brin-bawa-sepatu-buatan-sendiri-saat-temui-prabowo-mau-diproduksi-massal</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/sepatu-buatan-brin-evadetikcom-1785999841494_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Warga Bilang Pemotor Melintas di Trotoar Jl Sentul karena Putaran Balik Jauh</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:00:47 +0700</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Warga mengatakan pemotor melintas di trotoar Jalan Alternatif Sentul karena putaran balik jauh.</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606897/warga-bilang-pemotor-melintas-di-trotoar-jl-sentul-karena-putaran-balik-jauh</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/trotoar-di-jalan-alternatif-sentul-bogor-sering-dilewati-motor-sampai-rusak-rizkydetikcom-1785980261197_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Pria di Jakbar Kehilangan Motor Saat First Meet Wanita Kenalan Medsos</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:58:31 +0700</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Seorang pria menjadi korban curanmor di Kembangan, Jakbar. Sepeda motor pria itu diduga dibawa wanita saat pertemuan pertama (first meet) mereka.</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606895/pria-di-jakbar-kehilangan-motor-saat-first-meet-wanita-kenalan-medsos</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/seorang-pria-menjadi-korban-curanmor-di-kembangan-jakbar-sepeda-motor-pria-itu-diduga-dibawa-wanita-saat-pertemuan-pertama-fir-1785999460503_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Di Sekolah Pemilu Hijau, Kapolda Riau Dorong Green Policing untuk Green Election</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:54:29 +0700</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Kapolda Riau Irjen Herry Heryawan dukung Sekolah Pemilu Hijau KPU Riau. Ia menekankan pentingnya kolaborasi untuk demokrasi berkelanjutan.</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/melindungi-tuah-marwah/d-8606887/di-sekolah-pemilu-hijau-kapolda-riau-dorong-green-policing-untuk-green-election</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kapolda-riau-irjen-pol-herry-heryawan-menghadiri-peluncuran-sekolah-pemilu-hijau-di-kpu-riau-1785999184772_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Pemotor Tewas Usai Tabrak Trotoar di Jalan Juanda Depok</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:53:55 +0700</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Seorang pengendara motor berusia 29 tahun meninggal setelah kecelakaan tunggal menabrak trotoar di Jalan Juanda, Depok.</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606885/pemotor-tewas-usai-tabrak-trotoar-di-jalan-juanda-depok</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/tkp-kecelakaan-pemotor-tewas-usai-tabrak-trotoar-di-depok-1785999184753_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Kepala BGN Ungkap Kasus Keracunan MBG di Jayapura gegara Masak Terlalu Cepat</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:52:57 +0700</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>ANTARA</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Sejumlah siswa di Depapre, Papua, diduga keracunan setelah mengonsumsi MBG. BGN menyebut penyebabnya karena SPPG masak terlalu awal.</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606883/kepala-bgn-ungkap-kasus-keracunan-mbg-di-jayapura-gegara-masak-terlalu-cepat</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/kepala-bgn-sudaryono-1785937585412_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Ide Pilkada Tanpa Wakil, NasDem Singgung Banyak Kepala Daerah Kena OTT</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:52:55 +0700</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>NasDem menanggapi usulan pilkada tanpa wakil. Ia menekankan pentingnya kolaborasi antara kepala daerah dan wakil dalam pemerintahan.</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606882/ide-pilkada-tanpa-wakil-nasdem-singgung-banyak-kepala-daerah-kena-ott</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/12/14/kapoksi-komisi-ii-dpr-fraksi-nasdem-ujang-bey-1765691178496_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Detik-detik Nasabah di Cibitung Dirampok: Dibacok lalu Duit Rp 30 Juta Dicuri</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:47:21 +0700</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Seorang nasabah bank di Cibitung dirampok oleh komplotan bersenjata tajam, kehilangan Rp 30 juta. Polisi masih menyelidiki kasus ini.</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606870/detik-detik-nasabah-di-cibitung-dirampok-dibacok-lalu-duit-rp-30-juta-dicuri</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2019/06/24/f76d026c-9771-46e8-9200-8840de04f3ab_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Muzani Pastikan Sidang Tahunan MPR Digelar 14 Agustus, Ini Susunan Agendanya</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:47:06 +0700</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Ketua MPR RI, Ahmad Muzani, mengumumkan Sidang Tahunan MPR 2026 pada 14 Agustus. Agenda mencakup pidato kenegaraan dan laporan kinerja lembaga negara.</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606869/muzani-pastikan-sidang-tahunan-mpr-digelar-14-agustus-ini-susunan-agendanya</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/mpr-1785998788494_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Airlangga Ungkap Respons China soal Utang Kereta Cepat Ditanggung Kemenkeu</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:55:51 +0700</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>China disebut merespons baik upaya penyelesaian utang Whoosh yang akan dilakukan Indonesia.</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8606891/airlangga-ungkap-respons-china-soal-utang-kereta-cepat-ditanggung-kemenkeu</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/05/momen-airlangga-pamer-ekonomi-ri-tumbuh-lebih-tinggi-dari-as-china-1777977745953_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Alarm dari Kadin! Ekspor Nikel RI Terancam Hilang 5 Juta Ton</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:48:29 +0700</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Kadin Indonesia mengungkap dampak pemangkasan kuota nikel menjadi 260-270 juta ton, berpotensi hilangnya ekspor 3,5-5 juta ton. Kadin dorong kepastian RKAB.</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8606876/alarm-dari-kadin-ekspor-nikel-ri-terancam-hilang-5-juta-ton</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/07/21/nikel-indonesia-1753066004291_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>JHT hingga Pesangon Mulai Dibahas Pemerintah Jadi Alasan Buruh Batal Demo</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:28:40 +0700</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Presiden KSPI Said Iqbal memastikan tidak ada aksi buruh besar-besaran pada Agustus-September 2026.</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606831/jht-hingga-pesangon-mulai-dibahas-pemerintah-jadi-alasan-buruh-batal-demo</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/01/15/buruh-demo-dpr-keluhkan-kecilnya-kenaikan-ump-1768461540644_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Istana Buka Suara soal Utang Kereta Cepat Ditanggung Kementerian Keuangan</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:23:56 +0700</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Pihak istana buka suara soal penyelesaian utang Kereta Cepat Jakarta Bandung atau Whoosh yang akan diambil alih Kementerian Keuangan.</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8606826/istana-buka-suara-soal-utang-kereta-cepat-ditanggung-kementerian-keuangan</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/21/mensesneg-prasetyo-hadi-1784627991720_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Viral Dua JPO Rasuna Said Bikin Bingung, Konektivitas Antarmoda Jadi Sorotan</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:00:57 +0700</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Gilang Faturahman</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Dua JPO di Jalan H.R. Rasuna Said berdiri berdampingan, tetapi tak saling terhubung. Kondisi ini membuat sebagian pengguna transportasi umum harus memutar.</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8606610/viral-dua-jpo-rasuna-said-bikin-bingung-konektivitas-antarmoda-jadi-sorotan</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/konektivitas-jpo-rasuna-said-disorot-efisiensi-mobilitas-kawasan-bisnis-jadi-sorotan-1785989995354.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>IHSG Tertahan di Level 6.351</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:57:47 +0700</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Indeks Harga Saham Gabungan (IHSG) berakhir stagnan pada penutupan perdagangan sesi I hari ini, Kamis (6/8/2026).</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8606773/ihsg-tertahan-di-level-6-351</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/01/28/bei-terapkan-trading-halt-imbas-ihsg-anjlok-1769587530913_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Mendagri Ungkap 79 Pemda Butuh Tambahan Rp 14 T buat Bayar Pegawai</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:33:45 +0700</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Herdi Alif Al Hikam</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Menteri Dalam Negeri Tito Karnavian mengungkapkan pihaknya memetakan ada 79 pemerintah daerah yang butuh tambahan dana alokasi umum dari pemerintah pusat.</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606717/mendagri-ungkap-79-pemda-butuh-tambahan-rp-14-t-buat-bayar-pegawai</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/mendagri-wanti-wanti-kepala-daerah-jaga-integritas-demi-cegah-korupsi-1785894664987_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Rekening Raksasa Migas Iran Dibekukan Gegara Terlilit Utang Rp 304 T</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:30:04 +0700</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Rekening bank milik National Iranian Oil Company (NIOC) dibekukan oleh Bank of Industry and Mine milik pemerintah akibat utang yang terus membengkak.</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8606716/rekening-raksasa-migas-iran-dibekukan-gegara-terlilit-utang-rp-304-t</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2020/02/04/b21a4c0d-dca4-41fb-9380-5413e56fdc4e_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Said Iqbal Pastikan Tak Ada Demo Besar Buruh di Agustus-September</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:23:59 +0700</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Said Iqbal, Presiden KSPI, memastikan tidak ada aksi buruh besar di Agustus-September 2026. Meski demikian, ada empat tuntutan yang tetap diperjuangkan.</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606707/said-iqbal-pastikan-tak-ada-demo-besar-buruh-di-agustus-september</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/06/penasihat-khusus-presiden-bidang-ketenagakerjaan-dan-kesejahteraan-buruh-yang-juga-presiden-kspi-said-iqbal-1783315153767_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Sejarah di Liga Inggris! Manajer Baru Terbanyak dalam Semusim</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:00:20 +0700</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Liga Inggris musim 2026/27 catatkan sejarah. Itu adalah manajer baru terbanyak dalam semusim, ada sembilan lho!</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8606771/sejarah-di-liga-inggris-manajer-baru-terbanyak-dalam-semusim</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/14/andoni-iraola-1784017083641.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Singapura Vs Indonesia: Skuad Garuda Harus Lebih Kreatif</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:40:10 +0700</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Lucas Aditya</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia akan dijamu oleh Timnas Singapura dalam laga krusial di ajang Piala AFF 2026. Skuad Garuda dituntut untuk bermain lebih kreatif.</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8606685/singapura-vs-indonesia-skuad-garuda-harus-lebih-kreatif</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/03/garuda-dihajar-vietnam-0-3-mimpi-semifinal-kini-di-ujung-tanduk-1785773513300_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Kejuaraan Dunia di India: Alwi Farhan Fokus Main, Nggak Pikirin Venue</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:30:30 +0700</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Mercy Raya</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Alwi Farhan siap menghadapi tantangan besar Kejuaraan Dunia Bulutangkis yang digelar di India pada pertengahan Agustus ini.Alwi nggak mau pikirin venue.</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/raket/d-8606811/kejuaraan-dunia-di-india-alwi-farhan-fokus-main-nggak-pikirin-venue</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/22/alwi-farhan-1784694498208.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Real Madrid Mundur Beli Enzo Fernandez</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:20:30 +0700</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Beberapa bulan terakhir, Madrid rumornya mau beli Enzo Fernandez dari Chelsea. Namun sejauh ini, belum ada tawaran resmi yang masuk. Diyakini El Real mundur.</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8606682/real-madrid-mundur-beli-enzo-fernandez</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/22/enzo-fernandez-1784675213849.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Pesepakbola Thailand Meninggal Tersambar Petir di Lapangan</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:00:20 +0700</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Kabar duka dari Thailand. Pesepakbola di Liga 3 meninggal dunia akibat tersambar petir saat main di lapangan.</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/gila-bola/d-8606684/pesepakbola-thailand-meninggal-tersambar-petir-di-lapangan</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/05/08/ilustrasi-petir-1746676660826.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Arsenal Lebih Antusias Sambut Musim Baru, Berambisi Bikin Dinasti</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:40:40 +0700</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Okdwitya Karina Sari</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Setelah mengakhiri puasa panjang gelar Liga Inggris, Arsenal menatap musim 2026/2027 dengan lebih antusias. Arsenal punya ambisi menciptakan dinasti.</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8606583/arsenal-lebih-antusias-sambut-musim-baru-berambisi-bikin-dinasti</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/31/arsenal-1780241719681_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Head to Head Singapura Vs Indonesia: Garuda Unggul Atas The Lions</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:20:10 +0700</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Lucas Aditya</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Timnas Singapura akan berhadapan dengan Timnas Indonesia pada laga pamungkas Grup A Piala AFF 2026. Berikut catatan head to head kedua tim.</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8606628/head-to-head-singapura-vs-indonesia-garuda-unggul-atas-the-lions</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2018/11/09/ec0d1cd6-783b-4065-9b32-d41de7dc761c_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Van Dijk Bantu Leoni Lalui Masa-masa Sulit</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 12:00:35 +0700</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Mohammad Resha Pratama</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Tahun pertama sebagai pemain Liverpool tidaklah menyenangkan untuk Giovanni Leoni. Beruntung ada Virgil van Dijk yang menyemangati Leoni.</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8606431/van-dijk-bantu-leoni-lalui-masa-masa-sulit</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/giovanni-leoni-1785978207990_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>7 Kebiasaan Sepele yang Ternyata Bisa Merusak Kesehatan</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:13:56 +0700</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Beberapa kebiasaan yang terasa sepele dan tidak berbahaya nyatanya bisa berdampak buruk bagi kesehatan fisik dan mental dalam jangka panjang.</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>https://lifestyle.kompas.com/read/2026/08/06/141219720/7-kebiasaan-sepele-yang-ternyata-bisa-merusak-kesehatan</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/VxA_U17_Rqx0PKrJhw1giDHFFDA=/0x0:5145x3430/1200x675/filters:watermark(data/photo/2026/01/30/697c817ed68bb.png,0,-0,1)/data/photo/2025/09/05/68ba673443b91.jpg</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Tak Peduli Mau Dihukum Mati, Eks PM Bangladesh Tetap Ingin Pulang</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:13:57 +0700</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Eks PM Bangladesh yang digulingkan, Sheikh Hasina berencana untuk kembali ke negaranya dari pengasingan di India pada Desember.</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/global/read/2026/08/06/140000570/tak-peduli-mau-dihukum-mati-eks-pm-bangladesh-tetap-ingin-pulang</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/KqBi27DSy7i_XwV7Y5kK0f_RZ6Q=/79x22:1024x652/1200x675/filters:watermark(data/photo/2026/01/30/697c81ac46b81.png,0,-0,1)/data/photo/2024/08/05/66b0a34b78a2d.jpg</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>BGN Beri "Deadline" SPPG Penuhi SLHS, Paling Lambat 10 Agustus</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:13:58 +0700</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Kepala BGN memberi batas waktu hingga 10 Agustus 2026 bagi SPPG urus SLHS. Dapur yang tak penuhi standar akan ditutup permanen, kepala SPPG terancam dicopot.</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/06/13415551/bgn-beri-deadline-sppg-penuhi-slhs-paling-lambat-10-agustus</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/uXjDD9HgmL4W1tIqWolErz4__0I=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/07/29/6a69bd228d42b.jpeg</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I330"/>
+  <autoFilter ref="A1:I376"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 07:42 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$376</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$389</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I376"/>
+  <dimension ref="A1:I389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -18104,8 +18104,619 @@
         </is>
       </c>
     </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Lifestyle</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Benarkah kalori nasi merah lebih rendah dari nasi putih? Ini faktanya</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:25:42 +0700</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Anggapan bahwa nasi merah memiliki kalori lebih rendah dibandingkan nasi putih masih sering muncul, terutama di ...</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682388/benarkah-kalori-nasi-merah-lebih-rendah-dari-nasi-putih-ini-faktanya</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2020/07/02/DE121E3F-3DEF-4311-BACA-81FD21AB6D3F.jpeg</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Netanyahu Isyaratkan Siap Serang Iran Sendirian Tanpa AS</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:25:17 +0700</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Novi Christiastuti</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Netanyahu mengisyaratkan bahwa Israel dapat mengambil tindakan militer sepihak terhadap Iran, tanpa keterlibatan sekutu dekatnya AS.</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8606961/netanyahu-isyaratkan-siap-serang-iran-sendirian-tanpa-as</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/10/16/pm-israel-benjamin-netanyahu_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Kebakaran Gunung Bromo Belum Padam, Drone Water Spray dan Heli Dikerahkan</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:24:47 +0700</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>M Rofiq</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Petugas menggunakan helikopter dan drone water spray untuk padamkan kebakaran hutan di Gunung Bromo. Kebakaran mulai terkendali.</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606960/kebakaran-gunung-bromo-belum-padam-drone-water-spray-dan-heli-dikerahkan</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/proses-pemadaman-kebakaran-gunung-bromo-menggunakan-drone-water-spray-dan-heli-1785994028539_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Kapolda Riau: Green Policing Siap Menjadi Fondasi Menuju Green Election</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:22:16 +0700</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Mei Amelia R</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Kapolda Riau Irjen Herry Heryawan luncurkan Sekolah Pemilu Hijau, mengintegrasikan Green Policing untuk mendukung Green Election dan demokrasi berkelanjutan.</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/melindungi-tuah-marwah/d-8606947/kapolda-riau-green-policing-siap-menjadi-fondasi-menuju-green-election</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kapolda-riau-irjen-pol-herry-heryawan-menghadiri-peluncuran-sekolah-pemilu-hijau-di-kpu-riau-1785999184630_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Kebakaran di SDN Srengseng Jaksel Bersumber dari Gudang Buku</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:18:03 +0700</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Jabbar Ramdhani</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Kebakaran di SDN di Srengseng Sawah, Jagakarsa, Jakarta Selatan telah padam. Kebakaran terjadi di gudang penyimpanan buku.</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606938/kebakaran-di-sdn-srengseng-jaksel-bersumber-dari-gudang-buku</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kebakaran-di-sdn-di-srengseng-sawah-jagakarsa-jakarta-selatan-telah-padam-kebakaran-terjadi-di-gudang-penyimpanan-buku-dok-dam-1786000554778_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Purbaya Bakal Salurkan Rp 20 T Bantu Pemda Bayar Gaji ASN</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:27:17 +0700</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Kementerian Keuangan akan segera menyalurkan Rp 20,5 triliun kepada 490 pemerintah daerah untuk menjaga stabilitas keuangan daerah.</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606970/purbaya-bakal-salurkan-rp-20-t-bantu-pemda-bayar-gaji-asn</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/toko-online-lega-pemerintah-tunda-pajak-final-05-persen-1785929270093_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Kepala BRIN Pamer Teknologi Penyimpanan Gas, Bisa Pangkas Impor-Hemat Devisa</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:18:48 +0700</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Herdi Alif Al Hikam</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Ratusan peneliti Badan Riset dan Inovasi Nasional (BRIN) merapat ke Istana Kepresidenan, Jakarta Pusat.</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8606939/kepala-brin-pamer-teknologi-penyimpanan-gas-bisa-pangkas-impor-hemat-devisa</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kepala-brin-arif-satria-evadetikcom-1785997911603_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Pajak Toko Online Ditunda, Asosiasi e-Commerce Siap Ikuti Aturan</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:01:15 +0700</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Asosiasi E-commerce Indonesia (idEA) menanggapi keputusan pemerintah menunda penerapan pemungutan Pajak Penghasilan (PPh) Pasal 22 oleh marketplace.</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606898/pajak-toko-online-ditunda-asosiasi-e-commerce-siap-ikuti-aturan</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/02/24/ilustrasi-belanja-online-1771906901925_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Penjual Ikan Cupang Andalkan Live Streaming untuk Dongkrak Penjualan</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:00:13 +0700</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Andhika Prasetia</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Bisnis ikan cupang beradaptasi dengan pemasaran digital melalui live streaming. Strategi ini membantu menjaga penjualan di tengah perubahan tren pasar.</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8606596/penjual-ikan-cupang-andalkan-live-streaming-untuk-dongkrak-penjualan</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/penjual-ikan-cupang-andalkan-live-streaming-untuk-dongkrak-penjualan-1785989845605_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Mo Salah Pindah ke Turki, Diejek Bos Klub Arab Saudi</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:20:15 +0700</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Okdwitya Karina Sari</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Mohamed Salah segera diresmikan sebagai pemain baru klub Turki, Trabzonspor. Bos Al Kholood, Ben Harburg, mengejek kepindahan Mo Salah itu.</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8606774/mo-salah-pindah-ke-turki-diejek-bos-klub-arab-saudi</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/mohamed-salah-tiba-di-turki-siap-gabung-trabzonspor-1785933827411_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Alasan dan Penyebab Ruang Bahagia Cabut Gugatan terhadap Pemkot Solo</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:42:37 +0700</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Dalam sidang ini, pihak penggugat melalui kuasa hukumnya Asy' Adi Rouf kembali memohon untuk mencabut gugatan.</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/06/144210978/alasan-dan-penyebab-ruang-bahagia-cabut-gugatan-terhadap-pemkot-solo</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/UCkPHDXydNdPh5ppo5H-rM6uBrY=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/07/22/6a60ec53669f6.jpg</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Latihan di Beijing, Kunci Sukses Operasi Jantung LVAD Tanpa Perdarahan</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:42:37 +0700</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Tim dokter RSCM sempat terbang ke Beijing dan berlatih pada jantung babi sebelum sukses memasang LVAD tanpa perdarahan.</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>https://health.kompas.com/read/26H06142900268/latihan-di-beijing-kunci-sukses-operasi-jantung-lvad-tanpa-perdarahan</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/7eZpjBt-SmtKmcjwpV0fmldWL6w=/0x0:1280x853/1200x675/filters:watermark(data/photo/2026/01/30/697c819f9c086.png,0,-0,1)/data/photo/2026/08/05/6a7341b04fde6.jpeg</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Duduk Perkara Sekda Konawe Selatan Jadi Tersangka: Sempat Digerebek, Adik Terluka</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:42:38 +0700</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Duduk perkara Sekda Konawe Selatan jadi tersangka usai penggerebekan. Polisi ungkap kronologi insiden yang membuat adiknya terluka.</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/06/141358778/duduk-perkara-sekda-konawe-selatan-jadi-tersangka-sempat-digerebek-adik</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/wVZMC3im5NaV2QYn6qjXdAVk_p8=/217x34:1466x659/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a728e8559478.png</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I376"/>
+  <autoFilter ref="A1:I389"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 09:04 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$389</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$486</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I389"/>
+  <dimension ref="A1:I486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -18715,8 +18715,4567 @@
         </is>
       </c>
     </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Timnas 3x3 putri tampil di Singapore Series untuk persiapan AG 2026</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:50:13 +0700</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Timnas bola basket 3x3 putri Indonesia bersiap tampil untuk mengikuti FIBA 3x3 Women's Series Singapura 2026 pada ...</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682527/timnas-3x3-putri-tampil-di-singapore-series-untuk-persiapan-ag-2026</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/05/04/1000368703.jpg</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Polres Lumajang buat sekat bakar antisipasi karhutla TNBTS meluas</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:49:33 +0700</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Kepolisian Resor (Polres) Lumajang membuat sekat bakar darurat untuk mengantisipasi kebakaran hutan dan lahan ...</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682525/polres-lumajang-buat-sekat-bakar-antisipasi-karhutla-tnbts-meluas</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-15.20.11.jpeg</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Undian Kejuaraan Dunia 2026: Alwi Farhan berpotensi jumpa Shi Yu Qi</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:47:33 +0700</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Tunggal putra Indonesia Alwi Farhan berpotensi menghadapi unggulan pertama sekaligus juara bertahan asal China Shi Yu ...</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682524/undian-kejuaraan-dunia-2026-alwi-farhan-berpotensi-jumpa-shi-yu-qi</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/22/alwi-farhan-china-open.jpeg</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Konsultan: Eropa minati properti residensial dan komersial Indonesia</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:46:15 +0700</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Konsultan properti Knight Frank Indonesia menilai para pelaku usaha dari Uni Eropa atau EU meminati properti ...</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682523/konsultan-eropa-minati-properti-residensial-dan-komersial-indonesia</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1035.jpg</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Wapres Gibran tinjau langsung perkembangan pemulihan pascabencana di Aceh</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:43:51 +0700</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Wakil Presiden Gibran Rakabuming Raka mendengar penjelasan dari petugas Kementerian PU terkait pembangunan jembatan ...</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5682521/wapres-gibran-tinjau-langsung-perkembangan-pemulihan-pascabencana-di-aceh</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Kunker-Wapres-Gibran-ke-Aceh-060826-Rmd-4.jpg</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Korsel izinkan hak cipta untuk lagu yang dibuat dengan bantuan AI</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:43:34 +0700</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Korea Selatan akan mengizinkan pencipta untuk mendaftarkan hak cipta atas lagu yang dibuat dengan bantuan AI, asalkan ...</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682519/korsel-izinkan-hak-cipta-untuk-lagu-yang-dibuat-dengan-bantuan-ai</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/27/Bendera-Korea-Selatan_1.jpg</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Ketidakseimbangan bakteri baik usus picu gangguan perilaku anak</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:42:57 +0700</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Direktur Medical and Scientific Affairs, Danone Indonesia Dr. dr. Ray Wagiu Basrowi, MKK, FRSPH menyampaikan bahwa ...</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682515/ketidakseimbangan-bakteri-baik-usus-picu-gangguan-perilaku-anak</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/963bf01c-2c38-4cc2-914d-f1f457781e4e.jpeg</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>ESDM catat tambahan PNBP Rp20,98 miliar dari penegakan hukum</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:38:28 +0700</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Kementerian Energi dan Sumber Daya Mineral (ESDM) mencatat penambahan Penerimaan Negara Bukan Pajak (PNBP) sebesar ...</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682512/esdm-catat-tambahan-pnbp-rp2098-miliar-dari-penegakan-hukum</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/21/realisasi-devisa-ekspor-batu-bara-2825587.jpg</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Kepala BGN: 1.700 SPPG di daerah stunting tinggi siap beroperasi</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:38:15 +0700</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono menyebut 1.700 Satuan Pelayanan Pemenuhan Gizi (SPPG) di daerah dengan angka ...</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682508/kepala-bgn-1700-sppg-di-daerah-stunting-tinggi-siap-beroperasi</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/195031.jpg</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Bareskrim asistensi kasus penyelundupan 50 ton pasir timah di Belitung</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:32:33 +0700</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Direktorat Tindak Pidana Tertentu (Dittipidter) Bareskrim Polri menyatakan pihaknya akan mengasistensi penanganan kasus ...</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682507/bareskrim-asistensi-kasus-penyelundupan-50-ton-pasir-timah-di-belitung</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000087351.jpg</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Bappenas-Kemenbud kolaborasi kembangkan talenta seni budaya Indonesia</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:32:02 +0700</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Kementerian Perencanaan Pembangunan Nasional (PPN)/Badan Perencanaan Pembangunan Nasional (Bappenas) berkolaborasi ...</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682503/bappenas-kemenbud-kolaborasi-kembangkan-talenta-seni-budaya-indonesia</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-09.15.14-1.jpeg</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Pemerintah luncurkan Satu Data ZIS-DSKL perkuat integrasi data zakat</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:29:53 +0700</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Pemerintah melalui Kementerian Perencanaan Pembangunan Nasional/Badan Perencanaan Pembangunan Nasional (PPN/Bappenas), ...</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682495/pemerintah-luncurkan-satu-data-zis-dskl-perkuat-integrasi-data-zakat</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000176881.jpg</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Kemensos tangguhkan 1,49 juta penerima bansos terindikasi judi online</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:29:38 +0700</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial menangguhkan sebanyak 1.494.652 Keluarga Penerima Manfaat (KPM) Program Sembako yang terindikasi ...</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682491/kemensos-tangguhkan-149-juta-penerima-bansos-terindikasi-judi-online</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG-20260806-WA0004_1.jpg</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Zulhas: Ponpes dengan 1.000 lebih siswa asrama bisa bangun dapur MBG</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:28:46 +0700</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator Bidang Pangan Zulkifli Hasan (Zulhas) mengatakan pemerintah mengizinkan pondok pesantren (ponpes) ...</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682488/zulhas-ponpes-dengan-1000-lebih-siswa-asrama-bisa-bangun-dapur-mbg</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1E58581C-EB92-45A1-8253-849D0457835A.jpeg</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Menlu kawasan Pasifik berkumpul di Fiji jelang KTT</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:25:48 +0700</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Para menteri luar negeri dari 18 negara anggota Forum Kepulauan Pasifik (Pacific Islands Forum/PIF) berkumpul di Fiji ...</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682484/menlu-kawasan-pasifik-berkumpul-di-fiji-jelang-ktt</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2017/07/20170714pasifik.jpg</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>KemenHAM susun Perpres kepatuhan pelaku usaha dan HAM</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:25:14 +0700</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Kementerian Hak Asasi Manusia (KemenHAM) menyusun Rancangan Peraturan Presiden tentang Penilaian Kepatuhan Pelaku Usaha ...</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682483/kemenham-susun-perpres-kepatuhan-pelaku-usaha-dan-ham</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001221960.jpg</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>PSSI dukung penuh Gianni Infantino lanjutkan kepemimpinan di FIFA</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:24:56 +0700</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Persatuan Sepak Bola Seluruh Indonesia (PSSI) memberikan dukungan penuh terhadap Gianni Infantino untuk melanjutkan ...</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682481/pssi-dukung-penuh-gianni-infantino-lanjutkan-kepemimpinan-di-fifa</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/12/1000282681.jpg</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Legislator minta Polri semakin masif tindak judol pascatemuan PPATK</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:19:05 +0700</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Anggota Komisi III DPR RI Abdullah meminta Polri semakin masif menindak pelaku judi daring (judol) usai Pusat Pelaporan ...</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682480/legislator-minta-polri-semakin-masif-tindak-judol-pascatemuan-ppatk</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/09/Anggota_Komisi_III_DPR_RI_Abdullah_Foto_Dep_Alma20260409135732.jpeg</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Propam Jambi selidiki dugaan penipuan rekrutmen Polri Rp7,81 miliar</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:18:39 +0700</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Bidang Profesi dan Pengamanan (Bidpropam) Polda Jambi menyelidiki dugaan penipuan dalam rekrutmen Bintara Polri Tahun ...</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682479/propam-jambi-selidiki-dugaan-penipuan-rekrutmen-polri-rp781-miliar</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/369945.jpg</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Sri Mulyani Indrawati kembali duduki jabatan di Bank Dunia</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:17:29 +0700</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Bank Dunia menunjuk mantan Menteri Keuangan RI Sri Mulyani Indrawati sebagai Ketua Independen Asosiasi Pengembangan ...</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682473/sri-mulyani-indrawati-kembali-duduki-jabatan-di-bank-dunia</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/12/26/foto-terbaik-2025-2696596.jpg</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Kedubes Prancis resmikan Residensi Rimbaud perkuat pertukaran penulis</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:15:26 +0700</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Kedutaan Besar Prancis di Indonesia meluncurkan Residensi Rimbaud, program residensi sastra bilateral resiprokal ...</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682472/kedubes-prancis-resmikan-residensi-rimbaud-perkuat-pertukaran-penulis</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/03/28/Prancis.jpg</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Kemensos salurkan bansos triwulan III: PKH 7 juta KPM sembako 12 juta</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:10:44 +0700</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Kementerian Sosial mengakselerasi penyaluran bantuan sosial (bansos) Program Keluarga Harapan (PKH) dan Bantuan Pangan ...</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682471/kemensos-salurkan-bansos-triwulan-iii-pkh-7-juta-kpm-sembako-12-juta</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG-20260806-WA0004_1.jpg</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Nikita Bier resmi tinggalkan jabatan Kepala Produk di X</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:08:44 +0700</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Platform jejaring sosial, X, kembali harus kehilangan sosok pimpinan karena Nikita Bier yang sebelumnya dipercaya ...</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682468/nikita-bier-resmi-tinggalkan-jabatan-kepala-produk-di-x</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2023/07/30/WhatsApp-Image-2023-07-30-at-13.56.35.jpeg</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Prabowo terima paparan 15 stan riset unggulan BRIN</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:08:23 +0700</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menerima paparan hasil riset strategis Badan Riset dan Inovasi Nasional (BRIN) yang ...</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682465/prabowo-terima-paparan-15-stan-riset-unggulan-brin</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/27/IMG_3564.jpeg</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Wapres tinjau pemulihan infrastruktur pascabencana pembangunan di Aceh</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:06:27 +0700</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Wakil Presiden (Wapres) Gibran Rakabuming meninjau proses pemulihan infrastruktur dan layanan dasar pascabencana di ...</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682463/wapres-tinjau-pemulihan-infrastruktur-pascabencana-pembangunan-di-aceh</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/wapres-6.jpeg</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>DPR: Bantuan Rp20,5 triliun jaga fiskal 490 pemerintah daerah</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:00:03 +0700</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Anggota Komisi II DPR RI Rycko Menoza menyatakan rencana alokasi bantuan sebesar Rp20,5 triliun kepada 490 pemerintah ...</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682461/dpr-bantuan-rp205-triliun-jaga-fiskal-490-pemerintah-daerah</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/658f46bf-b25d-4563-90a3-9afd4efea3c6.jpeg</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Festival Raimuti 2026 di Manokwari</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:56:24 +0700</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Peserta mengikuti lomba perahu pada Festival Raimuti 2026 di Dermaga H Rahman Mansim, Manokwari, Papua Barat, Kamis ...</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5682457/festival-raimuti-2026-di-manokwari</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Festival-Raimuti-2026-di-Manokwari-682026-ci-4.jpg</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Presiden Iran sebut komunikasi dengan Motjaba Khamenei sangat sulit</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:55:25 +0700</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Presiden Iran Masoud Pezeshkian pada Rabu mengatakan bahwa komunikasi dengan Pemimpin Tertinggi Iran, Mojtaba Khamenei, ...</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682453/presiden-iran-sebut-komunikasi-dengan-motjaba-khamenei-sangat-sulit</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/21/thumbs_b_c_ed45147544be714dcdaa6c8ff91040f9.jpg</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Presiden Myanmar kunjungi Thailand guna peroleh legitimasi politik</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:53:41 +0700</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Presiden Myanmar Min Aung Hlaing pada Kamis melakukan kunjungan resmi ke Thailand selama dua hari, dan menurut pihak ...</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682449/presiden-myanmar-kunjungi-thailand-guna-peroleh-legitimasi-politik</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/10/XxjpbeE000254_20260410_PEPFN0A001A.jpg</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Toyota arahkan TEY-14 hasilkan aksi nyata dukung dekarbonisasi RI</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:53:05 +0700</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Toyota Indonesia mengarahkan penyelenggaraan Toyota Eco Youth (TEY) ke-14 tidak lagi sekadar menjadi kompetisi inovasi ...</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682447/toyota-arahkan-tey-14-hasilkan-aksi-nyata-dukung-dekarbonisasi-ri</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000177905.jpg</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Menpora inginkan muaythai Indonesia kejar emas di SEA Games 2027</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:48:41 +0700</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Menteri Pemuda dan Olahraga Erick Thohir menginginkan cabang olahraga muaythai Indonesia mampu meraih medali emas pada ...</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682445/menpora-inginkan-muaythai-indonesia-kejar-emas-di-sea-games-2027</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/17140b43-667b-44fd-916f-73ea39b039f1.jpeg</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Kejati pastikan tempuh banding terkait vonis bebas tiga anggota dewan</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:46:53 +0700</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Juru Bicara Kejaksaan Tinggi Nusa Tenggara Barat Harun Al Rasyid memastikan jaksa penuntut umum akan menempuh upaya ...</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682441/kejati-pastikan-tempuh-banding-terkait-vonis-bebas-tiga-anggota-dewan</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/sidang-putusan-gratifikasi-dprd-ntb.jpg</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Legislator: Identitas tunggal penting wujudkan pemilu berkualitas</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:44:28 +0700</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Anggota DPR RI Rycko Menoza mengatakan penerapan sistem identitas tunggal (single identity) menjadi salah satu langkah ...</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682439/legislator-identitas-tunggal-penting-wujudkan-pemilu-berkualitas</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/PHOTO-2026-08-06-11-21-27.jpg</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Bulog DKI-Banten masifkan pendistribusian beras premium ke toko retail</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:44:05 +0700</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Perusahaan Umum (Perum) Badan Urusan Logistik (Bulog) Kanwil DKI Jakarta dan Banten memasifkan pendistribusian ...</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682435/bulog-dki-banten-masifkan-pendistribusian-beras-premium-ke-toko-retail</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-13.33.24.jpeg</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Kemendikdasmen: Revitalisasi tembus pulau terluar setelah 21 tahun</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:43:15 +0700</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Kementerian Pendidikan Dasar dan Menengah (Kemendikdasmen) berhasil memperbaiki sarana dan prasarana layanan pendidikan ...</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682433/kemendikdasmen-revitalisasi-tembus-pulau-terluar-setelah-21-tahun</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000228793.jpg</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Jatim jajaki kerja sama industri-teknologi dengan perkapalan Tiongkok</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:42:53 +0700</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Jawa Timur menjajaki kerja sama sektor industri dan teknologi perkapalan dengan Republik Rakyat ...</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682429/jatim-jajaki-kerja-sama-industri-teknologi-dengan-perkapalan-tiongkok</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1329502.jpg</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Bareskrim respons kabar Anton Timbang hadiri pertemuan di Istana</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:42:14 +0700</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Direktorat Tindak Pidana Tertentu (Dittipidter) Bareskrim Polri merespons kabar tersangka kasus dugaan tersangka ...</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682425/bareskrim-respons-kabar-anton-timbang-hadiri-pertemuan-di-istana</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000087344.jpg</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Pertumbuhan pasar asuransi energi didorong ekspansi proyek migas</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:41:36 +0700</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>PT Asuransi Tugu Pratama Indonesia (Tugu Insurance) mencatat pasar asuransi energi nasional mengalami pertumbuhan ...</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682421/pertumbuhan-pasar-asuransi-energi-didorong-ekspansi-proyek-migas</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000454785.jpg</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>UOB Perkuat Bisnis Wealth Management melalui Kemitraan Distribusi Strategis dengan Allianz Global Investors</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:41:14 +0700</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>UOB Group menjalin kemitraan strategis dengan Allianz Global Investors (AGI). Melalui kemitraan ini, AGI akan ...</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682419/uob-perkuat-bisnis-wealth-management-melalui-kemitraan-distribusi-strategis-dengan-allianz-global-investors</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/UOB-x-Allianz-Global-Investors.jpg</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Disnakertrans Cianjur: Penempatan pekerja migran tekan pengangguran</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:41:09 +0700</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Dinas Tenaga Kerja dan Transmigrasi (Disnakertrans) Kabupaten Cianjur, Jawa Barat, mencatat program penempatan pekerja ...</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682415/disnakertrans-cianjur-penempatan-pekerja-migran-tekan-pengangguran</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/deni-ls.jpg</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Mendukbangga tinjau keluarga berisiko stunting di Pangkalpinang</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:36:17 +0700</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Menteri Kependudukan dan Pembangunan Keluarga (Mendukbangga) Republik Indonesia, Wihaji meninjau Keluarga Berisiko ...</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682411/mendukbangga-tinjau-keluarga-berisiko-stunting-di-pangkalpinang</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/mendukbangga3.jpg</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>WFP peringatkan El Nino berisiko perparah kerawanan pangan di Afrika</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:35:55 +0700</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Program Pangan Dunia (WFP) PBB pada Selasa (4/8) memperingatkan bahwa lebih dari 18 juta orang di seluruh Afrika Timur ...</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682408/wfp-peringatkan-el-nino-berisiko-perparah-kerawanan-pangan-di-afrika</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2024/07/24/XY37QCAE5VJUZO33FXDBHJYIO4_1.jpg</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Menbud sebut tradisi lisan bagian dari program pemajuan kebudayaan</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:32:42 +0700</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Menteri Kebudayaan Fadli Zon mengatakan bahwa tradisi lisan merupakan salah satu dari sepuluh obyek dari program ...</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682405/menbud-sebut-tradisi-lisan-bagian-dari-program-pemajuan-kebudayaan</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/05/Dongeng-akhir-pekan-untuk-mengisi-libur-sekolah-di-Bogor-050726-Arf-1.jpg</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Pemerintah fokus tingkatkan investasi dan pariwisata di Q3-2026</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:32:07 +0700</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator (Menko) Bidang Perekonomian Airlangga Hartarto mengatakan pemerintah fokus untuk meningkatkan ...</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682404/pemerintah-fokus-tingkatkan-investasi-dan-pariwisata-di-q3-2026</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_0441.jpeg</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Pemprov Maluku percepat penetapan kompensasi Blok Masela</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:29:20 +0700</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Maluku mempercepat penilaian dan penetapan kompensasi bagi masyarakat terdampak Proyek Strategis ...</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682403/pemprov-maluku-percepat-penetapan-kompensasi-blok-masela</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-10.29.25.jpeg</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Disbudpar Cianjur: Realisasi PAD sektor pariwisata capai 61 persen</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:28:51 +0700</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Dinas Kebudayaan dan Pariwisata (Disbudpar) Kabupaten Cianjur, Jawa Barat, mencatat realisasi Pendapatan Asli Daerah ...</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682399/disbudpar-cianjur-realisasi-pad-sektor-pariwisata-capai-61-persen</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/kadis-yudha.jpg</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>BRIN buat inovasi sepatu lokal harga Rp75 Ribu untuk Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:27:10 +0700</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Badan Riset dan Inovasi Nasional (BRIN) mengembangkan inovasi sepatu berbahan karet produksi lokal yang dibanderol ...</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682395/brin-buat-inovasi-sepatu-lokal-harga-rp75-ribu-untuk-sekolah-rakyat</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000034744.jpg</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>BRIN paparkan teknologi alternatif pengganti LPG ke Prabowo</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:27:02 +0700</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Badan Riset dan Inovasi Nasional (BRIN) akan memaparkan teknologi adsorbed natural gas (ANG) sebagai salah satu ...</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682392/brin-paparkan-teknologi-alternatif-pengganti-lpg-ke-prabowo</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000034746.jpg</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Ma'ruf Amin luncurkan buku dihadiri sejumlah bakal calon Ketum PBNU</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:25:00 +0700</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Wakil Presiden ke-13 RI Ma’ruf Amin meluncurkan buku berjudul Fikroh, Manhaj, dan Harakah Nahdhiyyah dalam ...</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682384/maruf-amin-luncurkan-buku-dihadiri-sejumlah-bakal-calon-ketum-pbnu</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000176845.jpg</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Kepala BGN Ungkap Penyebab Keracunan MBG di Papua: Masaknya Kecepetan</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:57:00 +0700</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono mengungkap penyebab banyaknya kasus keracunan dari program Makan Bergizi Gratis (MBG) di Papua.</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607145/kepala-bgn-ungkap-penyebab-keracunan-mbg-di-papua-masaknya-kecepetan</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kepala-badan-gizi-nasional-bgn-1786006514265_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Peserta Sidang Tahunan MPR 2026 Bakal Pakai PSL, Bukan Baju Adat</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:51:08 +0700</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Wakil Ketua MPR Eddy Soeparno mengungkapkan peserta sidang tahunan 2026 akan mengenakan pakaian sipil lengkap (PSL). Sidang digelar 14 Agustus.</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607138/peserta-sidang-tahunan-mpr-2026-bakal-pakai-psl-bukan-baju-adat</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/15/momen-pidato-perdana-prabowo-di-sidang-tahunan-mpr-1755233887571_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>MPR Kaji 3 Opsi Payung Hukum PPHN, Lewat Amandemen UUD atau Tap MPR</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:48:12 +0700</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Wakil Ketua MPR Eddy Soeparno mengungkapkan tiga opsi hukum untuk menetapkan PPHN. Termasuk amendemen UUD, TAP MPR, atau pembuatan undang-undang.</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607133/mpr-kaji-3-opsi-payung-hukum-pphn-lewat-amandemen-uud-atau-tap-mpr</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/eddy-soeparno-1786005656335_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Polisi Sisir Kali Licin Cari Potongan Kaki Korban Mutilasi di Depok</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:48:01 +0700</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Tim Resmob Polda Metro Jaya mencari potongan kaki korban mutilasi di Kali Licin, Depok. Tersangka Saepul mengaku membuangnya di lokasi tersebut.</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607132/polisi-sisir-kali-licin-cari-potongan-kaki-korban-mutilasi-di-depok</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/polisi-sisir-kali-licin-depok-mencari-potongan-kaki-korban-mutilasi-1786006025311_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>BRIN Pamerkan Robot hingga Kendaraan Otonom, Mensesneg: Tanda Indonesia Mampu</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:40:30 +0700</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menerima audiensi para peneliti dari Badan Riset dan Inovasi Nasional (BRIN) di Istana.</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607106/brin-pamerkan-robot-hingga-kendaraan-otonom-mensesneg-tanda-indonesia-mampu</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/brin-pamerkan-sejumlah-produk-di-istana-evadetikcom-1786005595142_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Lomba Foto LRT Hadirkan Hadiah Menarik, Ini Syaratnya</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:33:09 +0700</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>LRT Jabodebek menggelar Lomba Foto dengan hadiah menarik. Peserta dapat mengirimkan foto sesuai tema dan syarat yang ditentukan. Ikuti dan menangkan!</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607096/lomba-foto-lrt-hadirkan-hadiah-menarik-ini-syaratnya</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/lrt-jabodebek-1786005153603_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Mensesneg: Tak Ada Surpres Pergantian Kapolri</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:31:07 +0700</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Mensesneg Prasetyo Hadi menegaskan tidak ada surat presiden (surpres) terkait pergantian Kapolri Jenderal Listyo Sigit Prabowo.</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607089/mensesneg-tak-ada-surpres-pergantian-kapolri</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/21/mensesneg-prasetyo-hadi-1784627991634_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Demo Selesai, Sopir Angkot M44 Kembali Beroperasi dari Stasiun Tebet</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:30:30 +0700</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Adhfar Aulia Syuhada</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Sopir mikrolet M44 selesai demo di Balai Kota DKI Jakarta dan kembali beroperasi. Mereka menuntut evaluasi trayek JakLingko 48A yang berdampak pada pendapatan.</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607086/demo-selesai-sopir-angkot-m44-kembali-beroperasi-dari-stasiun-tebet</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/sopir-angkot-m44-kembali-beroperasi-dari-stasiun-tebet-usai-demo-1786004988741_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Disparekraf DKI Dorong Sport Tourism Lewat Jakarta Watersport Festival</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:27:09 +0700</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Jakarta Watersport Festival di Danau Sunter hadirkan olahraga air, hiburan, dan edukasi. Festival ini dorong kunjungan wisatawan dan dukung UMKM.</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607082/disparekraf-dki-dorong-sport-tourism-lewat-jakarta-watersport-festival</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/disparekraf-dki-dorong-sport-tourism-lewat-jakarta-watersport-festival-1786004753222_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Polisi Cokok 2 Pengedar di Jakbar, Sita Ribuan Tramadol hingga Vape Narkoba</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:26:29 +0700</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>Polsek Kembangan menangkap dua pengedar narkoba, RRF dan MS, di Cengkareng dan Grogol Petamburan. Barang bukti termasuk sabu dan vape berisi etomidate.</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607081/polisi-cokok-2-pengedar-di-jakbar-sita-ribuan-tramadol-hingga-vape-narkoba</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/polsek-kembangan-menangkap-dua-pengedar-narkoba-menyita-ribuan-tramadol-hingga-vape-etomidate-dan-sabu-1786004767626_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>DLH Siapkan Sanksi Perusahaan yang Diduga Bikin Air Kali Bekasi Hitam Bak Oli</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:25:21 +0700</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Rizky Adha Mahendra</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>DLH Kabupaten Bogor menyiapkan sanksi ke sejumlah perusahaan yang diduga membuat Kali Bekasi tercemar.</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607080/dlh-siapkan-sanksi-perusahaan-yang-diduga-bikin-air-kali-bekasi-hitam-bak-oli</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/video-air-kali-bekasi-berwarna-hitam-mirip-oli-bekas-viral-di-media-sosial-medsos-kualitas-air-tersebut-menurun-karena-ada-dug-1785929406139_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>22 Penumpang Ditolak Masuk Pesawat di Thailand Gegara Kejar Seleb</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:23:40 +0700</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Novi Christiastuti</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>Sebanyak 22 penumpang asal China dilarang masuk ke dalam pesawat maskapai Thai Airways menyusul insiden di Bandara Suvarnabhumi, Thailand.</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8607077/22-penumpang-ditolak-masuk-pesawat-di-thailand-gegara-kejar-seleb</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/ilustrasi-bandara-suvarnabhumi-1786004576201_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Kepala BGN Luruskan soal 13 Ribu SPPG, Begini Penjelasannya</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:21:49 +0700</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Kepala BGN Sudaryono menepis narasi yang menyebut pihaknya seolah-olah segera membuka 13 ribu dapur baru. Sudaryono menyebut SPPG akan dirilis secara bertahap.</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607075/kepala-bgn-luruskan-soal-13-ribu-sppg-begini-penjelasannya</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/tancap-gas-kepala-bgn-sudaryono-pecat-261-pegawai-bermasalah-1785138053252_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>BNN Tekankan Resiliensi Generasi Muda Hadapi Ancaman Narkotika</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:20:25 +0700</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Hana Nushratu Uzma</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>Kepala BNN Suyudi Ario Seto menekankan pentingnya resiliensi generasi muda dalam menolak narkotika. Acara di UNMA membahas dampak penyalahgunaan narkoba.</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607072/bnn-tekankan-resiliensi-generasi-muda-hadapi-ancaman-narkotika</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/bnn-1786004345632_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Polisi: Saepul Rencanakan Bunuh Pria di Depok demi Kuasai Harta Korban</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:16:26 +0700</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>Saepul (26) ditangkap setelah membunuh dan memutilasi K (51) di Depok. Ia berencana mencuri motor korban. Terancam hukuman mati.</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607056/polisi-saepul-rencanakan-bunuh-pria-di-depok-demi-kuasai-harta-korban</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/polisi-mengecek-temuan-mayat-mutilasi-di-tanah-kosong-pancoran-mas-kota-depok-1785896612343_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Pemprov Jateng &amp;amp; Kaltim Jalin Kerja Sama, Potensi Ekonomi Capai Rp 20,2 T</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:12:26 +0700</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>Jateng dan Kaltim jalin kerja sama dengan potensi ekonomi Rp 20,2 triliun. Fokus pada perdagangan, industri, dan proyek IKN untuk pembangunan berkelanjutan.</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/bangun-indonesia/d-8607044/pemprov-jateng-kaltim-jalin-kerja-sama-potensi-ekonomi-capai-rp-20-2-t</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/pemprov-jateng-kaltim-jalin-kerja-sama-potensi-ekonomi-capai-rp-202-t-1786003912828_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>DPD Soroti Dinamika Pusat-Daerah Lewat Buku, Ini Pesan Muzani</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:12:24 +0700</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Fara Difa Alfeni</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Dedi Iskandar menyerahkan buku DPD RI di Tengah Dinamika Kedaerahan kepada Ketua MPR RI. Buku ini mengulas peran DPD RI dalam sistem ketatanegaraan.</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607043/dpd-soroti-dinamika-pusat-daerah-lewat-buku-ini-pesan-muzani</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/mpr-1786002762003_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Prabowo Rapat Bareng Panglima TNI, Bahas Progres Jembatan hingga Listrik Desa</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:06:16 +0700</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menggelar rapat dengan Panglima TNI Jenderal TNI Agus Subiyanto dan jajarannya.</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607029/prabowo-rapat-bareng-panglima-tni-bahas-progres-jembatan-hingga-listrik-desa</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/prabowo-rapat-dengan-jajaran-pimpinan-tni-dok-setkab-1786003558651_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Melawan Perampok Bersajam, Nasabah di Cibitung Terluka di Tangan</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:04:42 +0700</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Wildan Noviansah</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>Seorang nasabah bank di Cibitung menjadi korban perampokan bersenjata, kehilangan Rp 30 juta dan terluka. Polisi masih memburu pelaku dan menyelidiki kasus ini.</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607027/melawan-perampok-bersajam-nasabah-di-cibitung-terluka-di-tangan</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2016/02/23/267bfe58-78ed-42ba-bbc5-e2e07b1df3b1_169.jpg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Penertiban Bangunan Liar di Tanah Abang Pulihkan Fungsi Drainase</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:00:35 +0700</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Ari Saputra</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>Pemkot Jakarta Pusat menertibkan bangunan semi permanen di atas saluran air di Tanah Abang. Langkah ini untuk menata kawasan dan memulihkan fungsi drainase.</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/foto-news/d-8606815/penertiban-bangunan-liar-di-tanah-abang-pulihkan-fungsi-drainase</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/normalisasi-drainase-95-bangunan-di-atas-saluran-phb-ditertibkan-1785996772444.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Menko Zulhas dan BGN Fokus SPPG di 3T, Targetkan Selesai Minggu Ini</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:59:35 +0700</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>Menko Pangan Zulkifli Hasan targetkan penyelesaian SPPG untuk makan bergizi gratis di daerah 3T, termasuk Papua, NTT, dan Maluku, dalam minggu ini.</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607020/menko-zulhas-dan-bgn-fokus-sppg-di-3t-targetkan-selesai-minggu-ini</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/menko-pangan-zulhas-hingga-kepala-bgn-sudaryono-menyampaikan-perkembangan-evaluasi-mbg-taufiqdetikcom-1786003142815_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Ahmad Muzani Pastikan MPR Matangkan Formulasi Hukum PPHN</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:53:42 +0700</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Dea Duta Aulia</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>MPR RI mematangkan Pokok-Pokok Haluan Negara (PPHN) sebagai pedoman nasional. Ahmad Muzani menekankan pentingnya konsensus untuk legitimasi PPHN.</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607003/ahmad-muzani-pastikan-mpr-matangkan-formulasi-hukum-pphn</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/mpr-1786002762084_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Kapolda Banten Ajak Warga Bikin Bak Tampung Air Hujan untuk Cadangan Kemarau</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:51:45 +0700</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Arief Ikhsanudin</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>Kapolda Banten Irjen Hengki mengusulkan pembangunan bak penampungan air hujan untuk atasi kekeringan.</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607000/kapolda-banten-ajak-warga-bikin-bak-tampung-air-hujan-untuk-cadangan-kemarau</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/kapolda-banten-1786002601261_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Zulhas Umumkan Ponpes Boleh Bikin SPPG, Ini Kriteria dan Syaratnya</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:51:35 +0700</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Taufiq Syarifudin</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>Zulhas mengumumkan pondok pesantren (ponpes) boleh membangun dapur Satuan Pelayanan Pemenuhan Gizi (SPPG) program Makan Bergizi Gratis (MBG).</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606999/zulhas-umumkan-ponpes-boleh-bikin-sppg-ini-kriteria-dan-syaratnya</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/jumpa-pers-mengenai-perbaikan-tata-kelola-program-makan-bergizi-gratis-taufiqdetikcom-1786002575542_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>BNN Hadiri Kuliah Umum Nasional di Universitas Majalengka</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:47:22 +0700</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Hana Nushratu Uzma</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>BNN menggelar Kuliah Umum di UNMA untuk tingkatkan literasi generasi muda terhadap ancaman narkotika. Fokus pada kesehatan dan karakter demi Indonesia Emas 2045</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606991/bnn-hadiri-kuliah-umum-nasional-di-universitas-majalengka</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/bnn-1786002372782_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Penampakan Senjata Api di Sekolah Jaksel, Kini Diusut Polisi</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:46:28 +0700</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>Penemuan senjata api di sekolah swasta Pondok Pinang, Jakarta Selatan, menggegerkan. Polisi sedang menyelidiki kepemilikan dan kronologi penemuan tersebut.</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606990/penampakan-senjata-api-di-sekolah-jaksel-kini-diusut-polisi</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/temuan-sejumlah-senjata-api-di-salah-satu-ruangan-yayasan-sekolah-swasta-di-pondok-pinang-jakarta-selatan-1786002238709_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Legislator Desak Usut Akar Masalah Terkait Nakes Diduga Hina Pasien BPJS</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:33:06 +0700</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>Anggota DPR Edy Wuryanto menyoroti dugaan nakes menghina pasien BPJS. Ia meminta evaluasi pelayanan kesehatan dan etika komunikasi tenaga medis di media sosial.</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8606978/legislator-desak-usut-akar-masalah-terkait-nakes-diduga-hina-pasien-bpjs</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/05/02/anggota-komisi-ix-dpr-ri-fraksi-pdip-edy-wuryanto-dok-istimewa-1746123691922_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Ketua Komisi XII DPR Dukung Perpres Atur Timah Masyarakat di Belitung</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:55:58 +0700</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>Ketua Komisi XII DPR Bambang Patijaya mendukung Pemerintah Pusat untuk menerbitkan Perpres sebagai legalitas timah masyarakat di Pulau Belitung.</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8607142/ketua-komisi-xii-dpr-dukung-perpres-atur-timah-masyarakat-di-belitung</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/03/04/ketua-komisi-xii-dpr-bambang-patijaya-1741099742550_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Penerima MBG Berpotensi Berkurang Imbas Temuan 6 Juta Data Ganda</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:51:48 +0700</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>Badan Gizi Nasional (BGN) mengungkapkan adanya potensi penurunan jumlah penerima program Makan Bergizi Gratis (MBG).</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8607140/penerima-mbg-berpotensi-berkurang-imbas-temuan-6-juta-data-ganda</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/22/kepala-bgn-sudaryono-1784715793188_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Danantara Dapat Tawaran Kempit Saham Bandara Madinah</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:48:45 +0700</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Herdi Alif Al Hikam</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>CEO Danantara Rosan Roeslani mengatakan pihaknya mendapatkan tawaran besar dari pemerintah Arab Saudi.</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8607136/danantara-dapat-tawaran-kempit-saham-bandara-madinah</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/16/ilustrasi-kantor-danantara-1784212600266_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Menperin Ungkap Pembiayaan buat Startup Turun hingga Rp 6,09 Triliun</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:41:56 +0700</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>Kementerian Perindustrian (Kemenperin) mencatat adanya penurunan pendanaan bagi startup nasional sepanjang tahun 2025.</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8607095/menperin-ungkap-pembiayaan-buat-startup-turun-hingga-rp-6-09-triliun</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/menteri-perindustrian-menperin-agus-gumiwang-kartasasmita-1786005067652_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Bos BGN Luruskan Isu 13 Ribu Dapur MBG Segera Dibuka</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:37:13 +0700</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>Kepala Badan Gizi Nasional (BGN) Sudaryono meluruskan terkait kabar 13.000 Satuan Pelayanan Pemenuhan Gizi (SPPG) akan segera dibuka.</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8607099/bos-bgn-luruskan-isu-13-ribu-dapur-mbg-segera-dibuka</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/27/tancap-gas-kepala-bgn-sudaryono-pecat-261-pegawai-bermasalah-1785138053252_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Kadin Minta Hilirisasi Jangan Cuma Jadi Mainan Konglomerat dan Asing</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:31:53 +0700</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Kadin Indonesia minta pemerintah beri ruang bagi pengusaha lokal dalam hilirisasi energi dan mineral.</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8607092/kadin-minta-hilirisasi-jangan-cuma-jadi-mainan-konglomerat-dan-asing</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/15/pembangunan-pabrik-di-kek-batang-pacu-pertumbuhan-investasi-nasional-1776264402935_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Pembangunan Tol Laut Teluk Jakarta Diharapkan Percepat Arus Logistik Nasional</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:30:24 +0700</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Pradita Utama</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>Pembangunan jalan akses pelabuhan di Teluk Jakarta ditargetkan mempercepat arus logistik sekaligus meningkatkan konektivitas pelabuhan. Begini progresnya.</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8607004/pembangunan-tol-laut-teluk-jakarta-diharapkan-percepat-arus-logistik-nasional</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/pembangunan-tol-laut-teluk-jakarta-diharapkan-percepat-arus-logistik-nasional-1786001253115_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>RI Berpeluang Jadi Raja Industri Protein Asia Tenggara</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:06:53 +0700</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>RI Berpeluang Jadi Raja Industri Protein Asia Tenggara, Sebesar Ini Potensinya</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8607030/ri-berpeluang-jadi-raja-industri-protein-asia-tenggara</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/04/09/meningkatnya-permintaan-telur-ayam-untuk-lebaran_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Janji Bulog Jaga Kualitas Beras Usai Dapat Margin Fee 7%</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:58:52 +0700</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>Bulog memastikan tambahan margin tersebut akan dikembalikan kepada masyarakat melalui peningkatan kualitas pelayanan dan mutu beras.</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8607018/janji-bulog-jaga-kualitas-beras-usai-dapat-margin-fee-7</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/06/29/bulog-tegaskan-tetap-serap-gabah-hasil-panen-petani-sepanjang-tahun-1782706837728_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Menanti Inklusifitas Angka Pertumbuhan Ekonomi</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:43:52 +0700</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>20detik Signature</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Apa strategi yang perlu disiapkan agar pertumbuhan itu lebih inklusif?</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606866/menanti-inklusifitas-angka-pertumbuhan-ekonomi</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/detiksore6-agustus-2026-1785998741725_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Pemerintah Selidiki Beras Fortifikasi Mahal, Klaim Gizi Bakal Diuji!</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:38:40 +0700</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Ilyas Fadilah</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>Pemerintah mendalami peredaran beras fortifikasi yang dijual dengan harga jauh lebih tinggi dibandingkan beras medium dan premium.</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606982/pemerintah-selidiki-beras-fortifikasi-mahal-klaim-gizi-bakal-diuji</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/08/27/kenaikan-harga-beras-1756283170846_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Said Iqbal Ungkap Alasan Buruh Batal Demo di Agustus</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:28:40 +0700</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>Presiden KSPI Said Iqbal memastikan tidak ada aksi buruh besar-besaran pada Agustus-September 2026.</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606831/said-iqbal-ungkap-alasan-buruh-batal-demo-di-agustus</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/01/15/buruh-demo-dpr-keluhkan-kecilnya-kenaikan-ump-1768461540644_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Singapura Vs Indonesia: Saatnya Garuda Menang di Kandang Singa</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:40:40 +0700</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Lucas Aditya</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>Timnas Indonesia sedang sulit menang di kandang Timnas Singapura. Kini, Garuda harus memperbaiki catatan itu demi tiket ke semifinal Piala AFF 2026.</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8606852/singapura-vs-indonesia-saatnya-garuda-menang-di-kandang-singa</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/12/23/singapura-vs-indonesia_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Lanny/Ester Awalnya Sering Tabrakan, Kini Siap Debut sebagai Pasangan Baru</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:30:35 +0700</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Mercy Raya</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>Jelang debut sebagai pasangan ganda putri, Lanny Tria Mayasari dan Ester Nurumi Tri Wardoyo mengaku sempat sering bertabrakan saat latihan.</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/raket/d-8607069/lanny-ester-awalnya-sering-tabrakan-kini-siap-debut-sebagai-pasangan-baru</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/lanny-tria-mayasari-ester-nurumi-tri-wardoyo-1786004143150_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Gianni Infantino Masih Aman Posisinya Sebagai Presiden FIFA</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:20:35 +0700</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>Gianni Infantino masih aman posisinya sebagai Presiden FIFA. Gianni percaya dirinya bisa lanjutkan periode keempat di pemilihan 2027 nanti.</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8606863/gianni-infantino-masih-aman-posisinya-sebagai-presiden-fifa</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/23/gianni-infantino-1784793685990.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Awas Menyesal Nanti Menyesal, Vinicius!</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:00:35 +0700</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Okdwitya Karina Sari</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Mantan bintang sekaligus direktur Real Madrid Predrag Mijatovic memperingatkan Vinicius Junior. Masa depan Vinicius lagi dipertanyakan menyusul rumor Arsenal.</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8606861/awas-menyesal-nanti-menyesal-vinicius</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/04/08/vinicius-junior-1775599794726_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Maraknya Tragedi Pesepakbola Tersambar Petir, Ada dari Indonesia</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:40:30 +0700</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>Beberapa tahun terakhir, tercatat tragedi pesepakbola-pesepakbola di dunia yang meninggal dunia karena tersambar petir. Ada dari Indonesia juga.</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/gila-bola/d-8606782/maraknya-tragedi-pesepakbola-tersambar-petir-ada-dari-indonesia</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/11/04/ilustrasi-hujan-petir-1762239904688.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Bawa Nama Negara, Alwi Farhan Enggan Pilih-pilih Turnamen</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 14:30:20 +0700</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Mercy Raya</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>Alwi Farhan menegaskan akan tampil maksimal di Kejuaraan Dunia, China Masters, dan Asian Games 2026. Ia tak mau pilih-pilih turnamen.</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/raket/d-8606909/bawa-nama-negara-alwi-farhan-enggan-pilih-pilih-turnamen</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/16/alwi-farhan-1784194208649_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Money</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Tugu Insurance Raup Laba Bersih Rp 480,29 Miliar, Naik 76,87 Persen Per Semester I 2026</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:04:02 +0700</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>Sejalan dengan itu, laba per saham (EPS) tercatat sebesar Rp 135, meningkat dari Rp 76 pada semester I-2025.</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/08/06/160346326/tugu-insurance-raup-laba-bersih-rp-48029-miliar-naik-7687-persen-per-semester</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/mbhBt5LU72-ZhS7UoDUurNBCkBs=/14x0:671x438/1200x675/filters:watermark(data/photo/2026/01/30/697c815e7ef28.png,0,-0,1)/data/photo/2025/11/01/6905f64557748.jpeg</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Penampakan Sepatu Lokal Rp 80.000 yang Mau Dipesan Prabowo</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:04:04 +0700</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>Kepala BRIN Arif Satria pamer sepatu lokal BRIN di Istana. Sepatu ini terbuat dari karet, harga Rp 80.000, dan dipesan juga oleh Presiden Prabowo.</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/08/06/15505431/penampakan-sepatu-lokal-rp-80000-yang-mau-dipesan-prabowo</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/RY8Sg6zLorYT1FJhOUh9l0lfYM4=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a744924700a2.jpg</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Polisi Tangkap Warga Cimahi Pembuat Video AI Manipulasi Gambar Presiden Prabowo, Sebar Konten Provokatif</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:04:05 +0700</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>Polda Jabar tangkap FG, warga Cimahi, karena manipulasi gambar Presiden Prabowo Subianto pakai AI di medsos dengan narasi provokatif.</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/08/06/153446578/polisi-tangkap-warga-cimahi-pembuat-video-ai-manipulasi-gambar-presiden</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/2u3Px-Lvy1c23FTkxGzd77N4Gco=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a744125a1976.jpg</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I389"/>
+  <autoFilter ref="A1:I486"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 09:34 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$486</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$527</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I486"/>
+  <dimension ref="A1:I527"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -23274,8 +23274,1935 @@
         </is>
       </c>
     </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Menaker ajak perguruan tinggi selaraskan kurikulum dengan industri</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:22:09 +0700</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli mengajak institusi pendidikan tinggi di seluruh Indonesia untuk semakin ...</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682591/menaker-ajak-perguruan-tinggi-selaraskan-kurikulum-dengan-industri</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_20260806_153622.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>OJK: Industri keuangan syariah bergerak ke arah yang lebih baik</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:21:27 +0700</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>Ketua Dewan Komisioner Otoritas Jasa Keuangan (OJK) Friderica Widyasari Dewi mengatakan industri keuangan syariah ...</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682588/ojk-industri-keuangan-syariah-bergerak-ke-arah-yang-lebih-baik</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/06/22/bsi-3.jpg</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Gubernur Koster tetapkan lima kawasan rendah emisi di Bali</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:20:44 +0700</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>Gubernur Bali Wayan Koster menetapkan proyek lima kawasan rendah emisi di Pulau Dewata yang tengah dipersiapkan sebagai ...</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682585/gubernur-koster-tetapkan-lima-kawasan-rendah-emisi-di-bali</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/70b440c1-582c-4718-a926-2d9a6b247016.jpeg</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Pemerintah monitor industri rentan PHK dan penciptaan lapangan kerja</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:20:20 +0700</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>Menteri Koordinator (Menko) Bidang Perekonomian Airlangga Hartarto memastikan pemerintah terus memonitor ...</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682583/pemerintah-monitor-industri-rentan-phk-dan-penciptaan-lapangan-kerja</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_0441.jpeg</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Uruguay sebut krisis Argentina-Brasil "kabar buruk" bagi Mercosur</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:16:33 +0700</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E491" t="inlineStr">
+        <is>
+          <t>Menteri Luar Negeri Uruguay Mario Lubetkin pada Rabu (5/8) mengatakan bahwa krisis diplomatik antara Argentina dan ...</t>
+        </is>
+      </c>
+      <c r="F491" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682576/uruguay-sebut-krisis-argentina-brasil-kabar-buruk-bagi-mercosur</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2016/06/20160626Mercosur.jpg</t>
+        </is>
+      </c>
+      <c r="I491" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Mensesneg membantah isu Surpres penggantian Kapolri</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:15:03 +0700</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E492" t="inlineStr">
+        <is>
+          <t>Menteri Sekretaris Negara (Menseneg) Prasetyo Hadi membantah isu mengenai penggantian Kapolri, dan ...</t>
+        </is>
+      </c>
+      <c r="F492" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682572/mensesneg-membantah-isu-surpres-penggantian-kapolri</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/sesneg.jpg</t>
+        </is>
+      </c>
+      <c r="I492" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Perkaya kualitas ajar, Menaker usul dosen cuti guna magang di industri</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:13:35 +0700</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E493" t="inlineStr">
+        <is>
+          <t>Menteri Ketenagakerjaan (Menaker) Yassierli mengusulkan gagasan inovatif kepada pimpinan perguruan tinggi untuk ...</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682569/perkaya-kualitas-ajar-menaker-usul-dosen-cuti-guna-magang-di-industri</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_20260806_154922.jpg.jpeg</t>
+        </is>
+      </c>
+      <c r="I493" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Selandia Baru luncurkan mata pelajaran baru berbasis industri</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:13:02 +0700</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E494" t="inlineStr">
+        <is>
+          <t>Selandia Baru pada Kamis (6/8) meluncurkan serangkaian mata pelajaran baru yang berbasis industri di tingkat sekolah ...</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682565/selandia-baru-luncurkan-mata-pelajaran-baru-berbasis-industri</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000020_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I494" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>TNBTS: "Drone water spray" dimaksimalkan tangani kebakaran di Bromo</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:13:01 +0700</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E495" t="inlineStr">
+        <is>
+          <t>Balai Besar Taman Nasional Bromo Tengger Semeru (TNBTS) menyatakan pemadaman kebakaran di kawasan Gunung Bromo ...</t>
+        </is>
+      </c>
+      <c r="F495" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682561/tnbts-drone-water-spray-dimaksimalkan-tanganikebakaran-di-bromo</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001402670.jpg</t>
+        </is>
+      </c>
+      <c r="I495" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Gulkarmat Jakpus bentuk Redkar di Senen percepat penanganan kebakaran</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:12:50 +0700</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E496" t="inlineStr">
+        <is>
+          <t>Suku Dinas Penanggulangan Kebakaran dan Penyelamatan (Gulkarmat) Jakarta Pusat membentuk Relawan Pemadam Kebakaran ...</t>
+        </is>
+      </c>
+      <c r="F496" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682560/gulkarmat-jakpus-bentuk-redkar-di-senen-percepat-penanganan-kebakaran</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2025/09/15/jakarta-fire-safety-challenge-2025-2623293.jpg</t>
+        </is>
+      </c>
+      <c r="I496" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>PBB sebut operasi militer Israel ganggu kehidupan warga sipil di Gaza</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:12:19 +0700</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E497" t="inlineStr">
+        <is>
+          <t>Operasi militer Israel di Jalur Gaza mengganggu kehidupan warga sipil, merusak tempat penampungan, serta meningkatkan ...</t>
+        </is>
+      </c>
+      <c r="F497" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682559/pbb-sebut-operasi-militer-israel-ganggu-kehidupan-warga-sipil-di-gaza</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/CjkinzN000004_20260806_CBMFN0A001.jpg</t>
+        </is>
+      </c>
+      <c r="I497" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>JATAM gugat Gubernur Sulteng soal limbah tailing di PTUN</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:10:54 +0700</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E498" t="inlineStr">
+        <is>
+          <t>Jaringan Advokasi Tambang (JATAM) Sulawesi Tengah menggugat Gubernur Sulawesi Tengah ke Pengadilan Tata Usaha Negara ...</t>
+        </is>
+      </c>
+      <c r="F498" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682555/jatam-gugat-gubernur-sulteng-soal-limbah-tailing-di-ptun</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/WhatsApp-Image-2026-08-06-at-16.14.33.jpeg</t>
+        </is>
+      </c>
+      <c r="I498" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Prabowo terima laporan capaian program TNI dukung pembangunan</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:10:48 +0700</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto menerima laporan perkembangan berbagai program strategis TNI yang mendukung pemerataan ...</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682553/prabowo-terima-laporan-capaian-program-tni-dukung-pembangunan</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000034773.jpg</t>
+        </is>
+      </c>
+      <c r="I499" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Wuling pamer dua model PHEV di GIIAS 2026</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:10:46 +0700</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/antaranewsdotcom</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>Memanfaatkan pameran otomotif Gaikindo Indonesia International Auto Show (GIIAS) 2026, Wuling motor (Wuling) ...</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>https://otomotif.antaranews.com/berita/5682551/wuling-pamer-dua-model-phev-di-giias-2026</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000503134.jpg</t>
+        </is>
+      </c>
+      <c r="I500" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Pemkot Jaktim gencarkan skrining TBC lewat CKG, sasar 77 ribu warga</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:08:29 +0700</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota (Pemkot) Jakarta Timur mulai menggencarkan program skrining Tuberkulosis (TBC) yang terintegrasi ...</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682548/pemkot-jaktim-gencarkan-skrining-tbc-lewat-ckg-sasar-77-ribu-warga</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/InShot_20260806_153422556.jpg</t>
+        </is>
+      </c>
+      <c r="I501" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>IESR sebut Program PLTS 100 GW dukung pertumbuhan ekonomi</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:05:42 +0700</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>Institute for Essential Services Reform (IESR) menyatakan program pembangunan pembangkit listrik tenaga surya (PLTS) ...</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682545/iesr-sebut-program-plts-100-gw-dukung-pertumbuhan-ekonomi</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_20260806_151807.jpg</t>
+        </is>
+      </c>
+      <c r="I502" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Pemprov Papua siap fasilitasi identifikasi jenazah korban PD II</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:05:33 +0700</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E503" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi (Pemprov) Papua menyatakan kesiapan memfasilitasi proses identifikasi kerangka jenazah korban ...</t>
+        </is>
+      </c>
+      <c r="F503" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682543/pemprov-papua-siap-fasilitasi-identifikasi-jenazah-korban-pd-ii</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1002069916.jpg</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Houthi klaim serangan rudal terhadap kapal minyak Saudi di Teluk Aden</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:05:28 +0700</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E504" t="inlineStr">
+        <is>
+          <t>Kelompok Houthi Yaman pada Rabu (5/8) menyatakan telah menargetkan sebuah kapal tanker minyak Arab Saudi dengan rudal ...</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682541/houthi-klaim-serangan-rudal-terhadap-kapal-minyak-saudi-di-teluk-aden</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/02/28/ilustrasi-rudal-Iran.jpg</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>BP BUMN-Danantara kawal ketat transformasi PT Pos Indonesia</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:04:41 +0700</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E505" t="inlineStr">
+        <is>
+          <t>BP BUMN dan Danantara melakukan monitoring rutin sebagai upaya mengawal proses transformasi PT Pos Indonesia agar ...</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682540/bp-bumn-danantara-kawal-ketat-transformasi-pt-pos-indonesia</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/29/WhatsApp-Image-2026-07-29-at-16.12.46.jpeg</t>
+        </is>
+      </c>
+      <c r="I505" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Pemerintah Aceh gencarkan BIAS 2026, tingkatkan kekebalan komunitas</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:04:14 +0700</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E506" t="inlineStr">
+        <is>
+          <t>ANTARA - Pemerintah Aceh mulai menggencarkan Bulan Imunisasi Anak Sekolah (BIAS) 2026 sepanjang Agustus. Penanggung ...</t>
+        </is>
+      </c>
+      <c r="F506" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5682499/pemerintah-aceh-gencarkan-bias-2026-tingkatkan-kekebalan-komunitas</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/Screenshot-2026-08-06-151427.jpg</t>
+        </is>
+      </c>
+      <c r="I506" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Kemenkes: 1 juta yang semula sehat terdeteksi hipertensi di CKG 2026</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:02:38 +0700</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E507" t="inlineStr">
+        <is>
+          <t>Kementerian Kesehatan dalam Cek Kesehatan Gratis (CKG) 2026 mendeteksi sekitar satu juta kasus baru hipertensi dari ...</t>
+        </is>
+      </c>
+      <c r="F507" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682536/kemenkes-1-juta-yang-semula-sehat-terdeteksi-hipertensi-di-ckg-2026</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/04/WhatsApp-Image-2026-08-04-at-19.09.09.jpeg</t>
+        </is>
+      </c>
+      <c r="I507" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Wamensos cek progres pembangunan SR Probolinggo hingga Polewali Mandar</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:02:01 +0700</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E508" t="inlineStr">
+        <is>
+          <t>Wakil Menteri Sosial Agus Jabo mengecek progres pembangunan Sekolah Rakyat di Probolinggo, Kuantan Singingi, dan ...</t>
+        </is>
+      </c>
+      <c r="F508" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682535/wamensos-cek-progres-pembangunan-sr-probolinggo-hingga-polewali-mandar</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000176885.jpg</t>
+        </is>
+      </c>
+      <c r="I508" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Legenda bulu tangkis akui wilayah timur masih kurang turnamen</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:59:07 +0700</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E509" t="inlineStr">
+        <is>
+          <t>Legenda bulu tangkis Indonesia Richard Mainaky mengatakan bibit atlet bulu tangkis di wilayah Timur Indonesia itu cukup ...</t>
+        </is>
+      </c>
+      <c r="F509" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G509" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682532/legenda-bulu-tangkis-akui-wilayah-timur-masih-kurang-turnamen</t>
+        </is>
+      </c>
+      <c r="H509" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/ImgResizer_Crop_1786005381193.jpg</t>
+        </is>
+      </c>
+      <c r="I509" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Kementerian PKP dan BPS perkuat data terkait bantuan perumahan</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:55:02 +0700</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E510" t="inlineStr">
+        <is>
+          <t>Kementerian Perumahan dan Kawasan Permukiman (PKP) menggandeng Badan Pusat Statistik (BPS) untuk memperkuat tata ...</t>
+        </is>
+      </c>
+      <c r="F510" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682529/kementerian-pkp-dan-bps-perkuat-data-terkait-bantuan-perumahan</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1037.jpg</t>
+        </is>
+      </c>
+      <c r="I510" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Potongan Kaki Korban Mutilasi Dicari, Saepul Ikut Dibawa ke Kali</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:22:01 +0700</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Devi Puspitasari</t>
+        </is>
+      </c>
+      <c r="E511" t="inlineStr">
+        <is>
+          <t>Tim Resmob Polda Metro Jaya melakukan penyisiran di Kali Licin, Depok, untuk mencari potongan kaki korban mutilasi. Tersangka Saepul hadir di lokasi.</t>
+        </is>
+      </c>
+      <c r="F511" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607221/potongan-kaki-korban-mutilasi-dicari-saepul-ikut-dibawa-ke-kali</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/polisi-melakukan-penyisiran-di-kali-licin-depok-untuk-mencari-potongan-kaki-korban-mutilasi-1786008041635_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I511" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Disdik Jaksel Siapkan Opsi PJJ Usai Kebakaran di SDN 04 Srengseng Sawah</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:15:59 +0700</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Brigitta Belia Permata Sari</t>
+        </is>
+      </c>
+      <c r="E512" t="inlineStr">
+        <is>
+          <t>Sudindik Wilayah I Jaksel menyiapkan skema pembelajaran hybrid bagi siswa pascakebakaran di SDN 04 Srengseng Sawah. PJJ disiapkan bagi siswa yang trauma.</t>
+        </is>
+      </c>
+      <c r="F512" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607200/disdik-jaksel-siapkan-opsi-pjj-usai-kebakaran-di-sdn-04-srengseng-sawah</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/sudindik-wilayah-i-jaksel-menyiapkan-skema-pembelajaran-hybrid-bagi-siswa-usai-kebakaran-yang-terjadi-di-sdn-04-srengseng-sawa-1786007697351_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I512" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Legislator Gerindra Dorong UMKM Palembang Lindungi Merek Usaha</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:12:23 +0700</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Annisa Sekar Melati</t>
+        </is>
+      </c>
+      <c r="E513" t="inlineStr">
+        <is>
+          <t>Partai Gerindra dorong UMKM Palembang untuk daftarkan merek dagang. Perlindungan hukum penting untuk daya saing dan keberlangsungan usaha.</t>
+        </is>
+      </c>
+      <c r="F513" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607184/legislator-gerindra-dorong-umkm-palembang-lindungi-merek-usaha</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/legislator-gerindra-kartika-sandra-desi-dorong-umkm-palembang-lindungi-merek-usaha-1786007525842.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I513" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Saksi Akui Tagihan PNBP Turun Rp 28 M Usai Beri Rp 1 M ke Eks Ketua Ombudsman</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:07:40 +0700</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Mulia Budi</t>
+        </is>
+      </c>
+      <c r="E514" t="inlineStr">
+        <is>
+          <t>Jaksa menghadirkan Tjia Peng Tjoan selaku Direktur PT Dinamika Sejahtera Mandiri sebagai saksi dalam sidang kasus suap mantan Ketua Ombudsman Hery Susanto.</t>
+        </is>
+      </c>
+      <c r="F514" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607168/saksi-akui-tagihan-pnbp-turun-rp-28-m-usai-beri-rp-1-m-ke-eks-ketua-ombudsman</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/sidang-eks-ketua-ombudsman-muliadetikcom-1785991541340_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I514" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Wamendagri Bima Arya Dorong DPRD Wujudkan Pembangunan Berkeadilan Ekologis</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:06:13 +0700</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E515" t="inlineStr">
+        <is>
+          <t>Wamendagri menekankan peran strategis DPRD dalam pembangunan berkeadilan ekologis. Legislator diharapkan optimalkan fungsi legislasi dan pengawasan.</t>
+        </is>
+      </c>
+      <c r="F515" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607165/wamendagri-bima-arya-dorong-dprd-wujudkan-pembangunan-berkeadilan-ekologis</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/wamendagri-bima-arya-dorong-dprd-wujudkan-pembangunan-berkeadilan-ekologis-1786007086451_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I515" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Polres OKI Genjot Kualitas Layanan Lewat Forum Konsultasi Publik Mandiri</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:05:18 +0700</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Inkana Putri</t>
+        </is>
+      </c>
+      <c r="E516" t="inlineStr">
+        <is>
+          <t>Polres OKI gelar Forum Konsultasi Publik 2026 untuk meningkatkan pelayanan publik. Kegiatan ini libatkan masyarakat &amp; berbagai elemen untuk evaluasi dan masukan</t>
+        </is>
+      </c>
+      <c r="F516" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/nyago-bumi-sriwijaya/d-8607162/polres-oki-genjot-kualitas-layanan-lewat-forum-konsultasi-publik-mandiri</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/polda-sumsel-1786006975157.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I516" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Ketum TP PKK Ajak Pelajar Biak Kenali Potensi Bahari untuk Cintai Tanah Air</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:03:47 +0700</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Rahmat Khairurizqi</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Ketua TP PKK Tri Tito Karnavian ajak pelajar Biak cintai Tanah Air melalui pendidikan karakter dan potensi bahari. Dukung program pemerintah untuk pendidikan.</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607160/ketum-tp-pkk-ajak-pelajar-biak-kenali-potensi-bahari-untuk-cintai-tanah-air</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/ketum-tp-pkk-ajak-pelajar-biak-kenali-potensi-bahari-untuk-cintai-tanah-air-1786007009183.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I517" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Korea Utara Tembakkan Proyektil Diduga Rudal Balistik, Jatuh ke Lautan</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:01:08 +0700</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Novi Christiastuti</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Korut terdeteksi menembakkan proyektil tak teridentifikasi pada Kamis (6/8) waktu setempat. Proyektil itu jatuh ke lautan di sebelah timur Semenanjung Korea.</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8607152/korea-utara-tembakkan-proyektil-diduga-rudal-balistik-jatuh-ke-lautan</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/06/27/korut-mengklaim-sukses-menguji-coba-rudal-yang-membawa-banyak-hulu-ledak-sekaligus_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I518" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>MPR Kaji 3 Opsi Payung Hukum PPHN, Lewat Amendemen UUD atau Tap MPR</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 15:48:12 +0700</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Anggi Muliawati</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Wakil Ketua MPR Eddy Soeparno mengungkapkan tiga opsi hukum untuk menetapkan PPHN. Termasuk amendemen UUD, Tap MPR, atau pembuatan undang-undang.</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607133/mpr-kaji-3-opsi-payung-hukum-pphn-lewat-amendemen-uud-atau-tap-mpr</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/eddy-soeparno-1786005656335_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I519" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>337 Saham Turun, IHSG Ditutup Melemah ke 6.343</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:23:56 +0700</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Indeks Harga Saham Gabungan (IHSG) ditutup melemah pada perdagangan hari ini. Pada penutupan pasar, IHSG tercatat di level 6.300.</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/bursa-dan-valas/d-8607228/337-saham-turun-ihsg-ditutup-melemah-ke-6-343</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/18/ihsg-anjlok-ke-zona-merah-bursa-saham-melemah-tajam-1779098741262_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I520" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Negara Raup Rp 20,9 M dari Lelang Batu Bara Sitaan</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:23:35 +0700</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Heri Purnomo</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Kementerian ESDM berhasil lelang 76.742 MT batu bara sitaan, menghasilkan PNBP Rp 20,9 miliar. Penegakan hukum dan pengelolaan aset negara diperkuat.</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8607227/negara-raup-rp-20-9-m-dari-lelang-batu-bara-sitaan</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/07/21/realisasi-devisa-ekspor-batu-bara-1784643932277_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I521" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Startup RI Urutan 6 Terbanyak di Dunia, tapi Mutunya Peringkat 45</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:14:12 +0700</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Andi Hidayat</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Menteri Perindustrian (Menperin), Agus Gumiwang Kartasasmita, menyebut Indonesia menjadi negara dengan jumlah startup terbesar ke enam dunia.</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G522" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8607187/startup-ri-urutan-6-terbanyak-di-dunia-tapi-mutunya-peringkat-45</t>
+        </is>
+      </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/08/08/ilustrasi-startup-atau-start-up_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I522" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Jembatan Kereta Api Jember Jalani Uji Beban Pascaperbaikan</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:00:45 +0700</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Tripa Ramadhan</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Jembatan kereta api di Jember jalani uji kekuatan usai perbaikan. Pengujian menggunakan dua lokomotif dilakukan untuk memastikan keselamatan perjalanan kereta.</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G523" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/foto-bisnis/d-8606568/jembatan-kereta-api-jember-jalani-uji-beban-pascaperbaikan</t>
+        </is>
+      </c>
+      <c r="H523" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/jembatan-kereta-api-jember-jalani-uji-beban-pascaperbaikan-1785989027280_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I523" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Mo Salah Pergi, Siapa yang Serba Nomor 1 di Liverpool Nanti?</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:00:10 +0700</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Afif Farhan</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Mohamed Salah dan Liverpool berpisah. Sejak kedatangan Salah, dirinya jadi pemain nomor 1 untuk urusan menjebol gawang lawan. Siapa yang bisa gantikannya?</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G524" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/foto-sepakbola/d-8606962/mo-salah-pergi-siapa-yang-serba-nomor-1-di-liverpool-nanti</t>
+        </is>
+      </c>
+      <c r="H524" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/05/mohamed-salah-1785943966122.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I524" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Viral Pengunjung Madiun Umbul Square Kecewa, Bayar Tiket Rp 20.000 Cuma Lihat Sedikit Satwa</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:34:46 +0700</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Video kekecewaan pengunjung Madiun Umbul Square viral karena bayar Rp 20.000 tapi lihat sedikit satwa. Ini kata Madiun Umbul Square dan BBKSDA Jatim</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G525" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/08/06/163415578/viral-pengunjung-madiun-umbul-square-kecewa-bayar-tiket-rp-20000-cuma-lihat</t>
+        </is>
+      </c>
+      <c r="H525" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/FRrWW69_C5OGEF4AD6DkUIqt4hs=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/06/6a743dbb0fd13.jpg</t>
+        </is>
+      </c>
+      <c r="I525" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Gubernur Kalsel Tagih Janji PLN Soal Pemadaman Listrik Berakhir Awal Agustus, Ternyata Molor</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:34:48 +0700</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Gubernur Kalsel menagih janji PLN terkait pemadaman listrik bergilir yang sebelumnya akan berakhir pada awal agustus. Ternyata molor.</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G526" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/08/06/161139378/gubernur-kalsel-tagih-janji-pln-soal-pemadaman-listrik-berakhir-awal</t>
+        </is>
+      </c>
+      <c r="H526" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/kq5cOLdimH3-4Pps8A5sESt7kFc=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/04/09/69d6e042e82e0.jpeg</t>
+        </is>
+      </c>
+      <c r="I526" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Regional</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Jadi Tersangka, Kabag Keuangan Setwan Ponorogo Diberhentikan Sementara dari PNS, Gaji 50 Persen</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:34:50 +0700</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Kompas Cyber Media</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Kabag Keuangan Setwan Ponorogo diberhentikan sementara dari statusnya sebagai PNS setelah ditetapkan menjadi tersangka korupsi</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G527" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/08/06/155645778/jadi-tersangka-kabag-keuangan-setwan-ponorogo-diberhentikan-sementara-dari</t>
+        </is>
+      </c>
+      <c r="H527" t="inlineStr">
+        <is>
+          <t>https://asset.kompas.com/crops/_gWtM5mJDhF_q9c6SCOILYLS7XE=/0x0:0x0/1200x675/filters:watermark(data/photo/2026/01/30/697c815a5f0b9.png,0,-0,1)/data/photo/2026/08/05/6a73255eca5c8.jpg</t>
+        </is>
+      </c>
+      <c r="I527" t="inlineStr">
+        <is>
+          <t>Kompas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I486"/>
+  <autoFilter ref="A1:I527"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-06 23:52 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1181</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1138"/>
+  <dimension ref="A1:I1181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -53924,8 +53924,2029 @@
         </is>
       </c>
     </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>KPK dalami pemberian Blueray Cargo kepada pegawai Bea Cukai</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:59:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1139" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>Komisi Pemberantasan Korupsi (KPK) mendalami pemberian sejumlah uang dari PT Blueray Cargo kepada pegawai Direktorat ...</t>
+        </is>
+      </c>
+      <c r="F1139" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1139" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683435/kpk-dalami-pemberian-blueray-cargo-kepada-pegawai-bea-cukai</t>
+        </is>
+      </c>
+      <c r="H1139" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/pemeriksaan-iskandar-sitorus-sebagai-saksi-2835524.jpg</t>
+        </is>
+      </c>
+      <c r="I1139" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>KPK dalami selisih uang yang dikembalikan Menhut dari Suhardiman Amby</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:54:25 +0700</t>
+        </is>
+      </c>
+      <c r="D1140" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>ANTARA - Komisi Pemberantasan Korupsi (KPK) mendalami selisih uang yang dikembalikan Menteri Kehutanan Raja Juli Antoni ...</t>
+        </is>
+      </c>
+      <c r="F1140" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1140" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5683413/kpk-dalami-selisih-uang-yang-dikembalikan-menhut-dari-suhardiman-amby</t>
+        </is>
+      </c>
+      <c r="H1140" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/KPK-DALAMI-SELISIH-UANG-YANG-DIKEMBALIKAN-MENHUT-DARI-SUHARDIMAN-AMBY.jpg</t>
+        </is>
+      </c>
+      <c r="I1140" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>Warga keluhkan dampak revitalisasi Kali Cakung Lama di Kelapa Gading</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:54:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1141" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>Warga Kampung Rawa Indah, RT 04/03, Kelurahan Pegangsaan Dua, Kecamatan Kelapa Gading, Jakarta Utara, mengeluhkan ...</t>
+        </is>
+      </c>
+      <c r="F1141" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1141" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683433/warga-keluhkan-dampak-revitalisasi-kali-cakung-lama-di-kelapa-gading</t>
+        </is>
+      </c>
+      <c r="H1141" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_4288.jpeg</t>
+        </is>
+      </c>
+      <c r="I1141" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>Dallas Mavericks perpanjang kontrak Naji Marshall</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:47:51 +0700</t>
+        </is>
+      </c>
+      <c r="D1142" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>Dallas Mavericks memperpanjang kontrak forward Naji Marshall setelah pemain berumur 28 tahun itu mencatatkan musim ...</t>
+        </is>
+      </c>
+      <c r="F1142" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1142" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683429/dallas-mavericks-perpanjang-kontrak-naji-marshall</t>
+        </is>
+      </c>
+      <c r="H1142" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000474637.jpg</t>
+        </is>
+      </c>
+      <c r="I1142" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Hoki putra-putri Indonesia segrup dengan Jepang pada Asian Games 2026</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:43:13 +0700</t>
+        </is>
+      </c>
+      <c r="D1143" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>Tim nasional hoki lapangan Indonesia, baik putra maupun putri, berada satu grup atau pul dengan tuan rumah Jepang pada ...</t>
+        </is>
+      </c>
+      <c r="F1143" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1143" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683423/hoki-putra-putri-indonesia-segrup-dengan-jepang-pada-asian-games-2026</t>
+        </is>
+      </c>
+      <c r="H1143" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/04/26/Tim-hoki-putri-Indonesia-kalahkan-Singapura-260626-fzn-12.jpg</t>
+        </is>
+      </c>
+      <c r="I1143" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Komunikasi ATR/BPN baik dan meraih Popular Government Institutions</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:42:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1144" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>Kementerian Agraria dan Tata Ruang (ATR)/Badan Pertanahan Nasional (BPN) meraih Popular Government Institutions Award ...</t>
+        </is>
+      </c>
+      <c r="F1144" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1144" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683420/komunikasi-atr-bpn-baik-dan-meraih-popular-government-institutions</t>
+        </is>
+      </c>
+      <c r="H1144" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_20260806_232006.jpg</t>
+        </is>
+      </c>
+      <c r="I1144" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>PB SEMMI respons isu Surpres ganti Kapolri: Kinerja Listyo Sigit baik</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:37:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1145" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>Pengurus Besar Serikat Mahasiswa Muslimin Indonesia (PB SEMMI) merespon isu adanya Surat Presiden (Supres) tentang ...</t>
+        </is>
+      </c>
+      <c r="F1145" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1145" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683419/pb-semmi-respons-isu-surpres-ganti-kapolri-kinerja-listyo-sigit-baik</t>
+        </is>
+      </c>
+      <c r="H1145" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/05/1000087296.jpg</t>
+        </is>
+      </c>
+      <c r="I1145" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Pemkot memetakan potensi kerawanan tawuran dan konflik sosial di Jakut</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:34:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1146" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota (Pemkot) Jakarta Utara (Jakut) memetakan potensi kerawanan tawuran dan konflik sosial lewat forum ...</t>
+        </is>
+      </c>
+      <c r="F1146" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1146" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683416/pemkot-memetakan-potensi-kerawanan-tawuran-dan-konflik-sosial-di-jakut</t>
+        </is>
+      </c>
+      <c r="H1146" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1771904152_ae8bf4453e35621f9af3-2.jpeg</t>
+        </is>
+      </c>
+      <c r="I1146" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>KPI ajak masyarakat kritis atas informasi tak valid di media sosial</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:32:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1147" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>Komisi Penyiaran Indonesia (KPI) mengajak kepada masyarakat untuk bersikap kritis terhadap maraknya informasi tidak ...</t>
+        </is>
+      </c>
+      <c r="F1147" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1147" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683415/kpi-ajak-masyarakat-kritis-atas-informasi-tak-valid-di-media-sosial</t>
+        </is>
+      </c>
+      <c r="H1147" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1001299202.jpg</t>
+        </is>
+      </c>
+      <c r="I1147" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Warga Jakbar diimbau lakukan deteksi dini kanker payudara</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:20:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1148" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Jakarta Barat (Pemkot Jakbar) menegaskan pentingnya deteksi dini sebagai upaya preventif dan ...</t>
+        </is>
+      </c>
+      <c r="F1148" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1148" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683409/warga-jakbar-diimbau-lakukan-deteksi-dini-kanker-payudara</t>
+        </is>
+      </c>
+      <c r="H1148" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/IMG_20260806_224733.v1.jpg</t>
+        </is>
+      </c>
+      <c r="I1148" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Menkum menargetkan kerja sama dengan 1.000 LBH di 2027</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:19:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1149" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>Menteri Hukum (Menkum) Supratman Andi Agtas menargetkan kerja sama dengan 1.000 lembaga bantuan hukum (LBH) atau ...</t>
+        </is>
+      </c>
+      <c r="F1149" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1149" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683408/menkum-menargetkan-kerja-sama-dengan-1000-lbh-di-2027</t>
+        </is>
+      </c>
+      <c r="H1149" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000473336.jpg</t>
+        </is>
+      </c>
+      <c r="I1149" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Menang dramatis, Persebaya Surabaya juara Piala Presiden 2026</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:16:10 +0700</t>
+        </is>
+      </c>
+      <c r="D1150" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>Pesepak bola Persebaya Surabaya Ramadhan Sananta berselebrasi setelah mencetak gol ke gawang Persib Bandung pada final ...</t>
+        </is>
+      </c>
+      <c r="F1150" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1150" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/foto/5683407/menang-dramatis-persebaya-surabaya-juara-piala-presiden-2026</t>
+        </is>
+      </c>
+      <c r="H1150" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/Final-Piala-Presiden-2026-060826-rzl-1.jpg</t>
+        </is>
+      </c>
+      <c r="I1150" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Pemerintah sasar cakupan 5G nasional 2029 optimalkan pemanfaatan AI</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:13:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1151" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>Kementerian Komunikasi dan Digital (Kemkomdigi) menyasar agar cakupan 5G nasional bisa terwujud di 2029, sehingga ke ...</t>
+        </is>
+      </c>
+      <c r="F1151" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1151" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683401/pemerintah-sasar-cakupan-5g-nasional-2029-optimalkan-pemanfaatan-ai</t>
+        </is>
+      </c>
+      <c r="H1151" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/InShot_20260806_230301926.jpg</t>
+        </is>
+      </c>
+      <c r="I1151" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Diego Forlan jadi pelatih interim timnas Uruguay</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:10:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1152" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>Legenda sepak bola Uruguay, Diego Forlan ditunjuk sebagai pelatih interim tim nasional Uruguay setelah Marcelo Bielsa ...</t>
+        </is>
+      </c>
+      <c r="F1152" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1152" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683400/diego-forlan-jadi-pelatih-interim-timnas-uruguay</t>
+        </is>
+      </c>
+      <c r="H1152" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/06/1000042734.jpg</t>
+        </is>
+      </c>
+      <c r="I1152" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>Terkini</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Gubernur Khofifah lepas kontingen Pramuka Jatim ke Jambore Nasional</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:08:14 +0700</t>
+        </is>
+      </c>
+      <c r="D1153" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>ANTARA - Gubernur Jawa Timur, Khofifah Indar Parawansa, menanamkan semangat heroisme bagi kontingen Pramuka asal ...</t>
+        </is>
+      </c>
+      <c r="F1153" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1153" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5683381/gubernur-khofifah-lepas-kontingen-pramuka-jatim-ke-jambore-nasional</t>
+        </is>
+      </c>
+      <c r="H1153" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/GUBERNUR-KHOFIFAH-LEPAS-KONTINGEN-PRAMUKA-JATIM-KE-JAMBORE-NASIONAL.jpg</t>
+        </is>
+      </c>
+      <c r="I1153" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Realisasi investasi Jakarta serap 289 ribu tenaga kerja</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:30:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1154" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>Realisasi investasi Jakarta pada semester I 2026 yang mencapai Rp173,6 triliun menyerap 289 ribu tenaga kerja, terdiri ...</t>
+        </is>
+      </c>
+      <c r="F1154" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1154" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5683152/realisasi-investasi-jakarta-serap-289-ribu-tenaga-kerja</t>
+        </is>
+      </c>
+      <c r="H1154" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/07/07/bursa-kerja-di-jakarta-2817824.jpg</t>
+        </is>
+      </c>
+      <c r="I1154" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>Top News</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Kronologi temuan 995 pucuk senjata api di sekolah swasta Jaksel</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 18:00:52 +0700</t>
+        </is>
+      </c>
+      <c r="D1155" t="inlineStr">
+        <is>
+          <t>antaranews.com</t>
+        </is>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>Tim kuasa hukum sekolah swasta di kawasan Pondok Pinang, Kebayoran Lama, Jakarta Selatan mengungkap kronologi temuan ...</t>
+        </is>
+      </c>
+      <c r="F1155" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1155" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5682835/kronologi-temuan-995-pucuk-senjata-api-di-sekolah-swasta-jaksel</t>
+        </is>
+      </c>
+      <c r="H1155" t="inlineStr">
+        <is>
+          <t>https://cdn.antaranews.com/cache/800x533/2026/08/07/1001014922.jpg</t>
+        </is>
+      </c>
+      <c r="I1155" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Pria di Jakut Tersengat Listrik Saat Mau Curi Kabel Gardu, Alami Luka Bakar</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:42:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1156" t="inlineStr">
+        <is>
+          <t>Antara</t>
+        </is>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>Seorang pria berinisial SD tersengat listrik saat mencoba mencuri kabel di gardu, mengalami luka bakar parah dan dirawat di RS Polri Kramat Jati.</t>
+        </is>
+      </c>
+      <c r="F1156" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1156" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607786/pria-di-jakut-tersengat-listrik-saat-mau-curi-kabel-gardu-alami-luka-bakar</t>
+        </is>
+      </c>
+      <c r="H1156" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2025/05/07/tangan-tersengat-listrik-1746608472483_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1156" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Pemerintah Renovasi Sekretariat LVRI, Bedah Rumah Veteran di 19 Provinsi</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:42:24 +0700</t>
+        </is>
+      </c>
+      <c r="D1157" t="inlineStr">
+        <is>
+          <t>Kadek Melda Luxiana</t>
+        </is>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>Kementerian Pertahanan merenovasi 9 sekretariat LVRI dan 52 rumah veteran di 19 provinsi. Program ini wujud penghormatan negara kepada pejuang bangsa.</t>
+        </is>
+      </c>
+      <c r="F1157" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1157" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607785/pemerintah-renovasi-sekretariat-lvri-bedah-rumah-veteran-di-19-provinsi</t>
+        </is>
+      </c>
+      <c r="H1157" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/pemerintah-renovasi-sekertariat-lvri-dan-rumah-veteran-di-19-provinsi-dok-istimewa-1786034404798_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1157" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Geger Mayat dalam Bagasi Mobil di Grobogan, Diduga Bos Konter HP yang Hilang</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:16:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1158" t="inlineStr">
+        <is>
+          <t>Ardian Dwi Kurnia</t>
+        </is>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>Warga Gubug, Grobogan, dikejutkan penemuan mayat dalam bagasi mobil. Diduga korban merupakan bos konten HP yang hilang di Ambarawa</t>
+        </is>
+      </c>
+      <c r="F1158" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1158" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607777/geger-mayat-dalam-bagasi-mobil-di-grobogan-diduga-bos-konter-hp-yang-hilang</t>
+        </is>
+      </c>
+      <c r="H1158" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2022/08/23/penemuan-mayat-wanita-duduk-di-melaya_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1158" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>BRIN: Presiden Beri Atensi Riset Pengelolaan Sampah hingga Genteng dari Limbah</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:41:57 +0700</t>
+        </is>
+      </c>
+      <c r="D1159" t="inlineStr">
+        <is>
+          <t>Eva Safitri</t>
+        </is>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto apresiasi inovasi BRIN, termasuk teknologi pengelolaan sampah dan genteng ramah lingkungan. Kerja sama uji coba juga sedang dibangun.</t>
+        </is>
+      </c>
+      <c r="F1159" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1159" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607760/brin-presiden-beri-atensi-riset-pengelolaan-sampah-hingga-genteng-dari-limbah</t>
+        </is>
+      </c>
+      <c r="H1159" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/presiden-prabowo-melihat-hasil-riset-brin-cahyo-biro-pers-media-dan-informasi-sekretariat-presiden-1786030862950.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1159" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Penjaga hingga Pembuang Sampah di TPS Liar Jaktim Didenda Rp 5 Juta</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:29:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1160" t="inlineStr">
+        <is>
+          <t>Rolando Fransiscus Sihombing</t>
+        </is>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Jakarta menindak tegas penimbunan sampah ilegal di Kramat Jati. Tiga pelaku dikenai sanksi denda administratif untuk mencegah pelanggaran serupa.</t>
+        </is>
+      </c>
+      <c r="F1160" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1160" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607751/penjaga-hingga-pembuang-sampah-di-tps-liar-jaktim-didenda-rp-5-juta</t>
+        </is>
+      </c>
+      <c r="H1160" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/pemprov-dki-periksa-tps-liar-di-jaktim-1786030130768_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1160" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Mobil Terbakar di Tol Dalam Kota, Lalin Arah Cawang Macet Malam Ini</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:08:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1161" t="inlineStr">
+        <is>
+          <t>Kadek Melda Luxiana</t>
+        </is>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>Sebuah mobil Toyota Rush terbakar di Tol Dalam Kota arah Cawang, menyebabkan kemacetan. Api sudah padam, namun proses pendinginan masih berlangsung.</t>
+        </is>
+      </c>
+      <c r="F1161" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1161" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8607745/mobil-terbakar-di-tol-dalam-kota-lalin-arah-cawang-macet-malam-ini</t>
+        </is>
+      </c>
+      <c r="H1161" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2024/11/13/ilustrasi-api_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1161" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Jurus Bank Jago Genjot Nasabah</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:39:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1162" t="inlineStr">
+        <is>
+          <t>Amanda Christabel</t>
+        </is>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>Bank Jago menggandeng Bibit &amp; Stockbit sejak 2021, untuk memberikan opsi investasi di dalam layanan perbankan digital.</t>
+        </is>
+      </c>
+      <c r="F1162" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1162" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8607783/jurus-bank-jago-genjot-nasabah</t>
+        </is>
+      </c>
+      <c r="H1162" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2021/04/15/bank-jago_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1162" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Pedestrian Deck Dukuh Atas: Ketika Kota Dibangun dari Langkah Kaki</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:00:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1163" t="inlineStr">
+        <is>
+          <t>Shafira Cendra Arini</t>
+        </is>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>Salah satu wujudnya di kawasan Dukuh Atas yang dirancang sebagai simpul transportasi terpadu dengan enam moda transportasi publik.</t>
+        </is>
+      </c>
+      <c r="F1163" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1163" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8607770/pedestrian-deck-dukuh-atas-ketika-kota-dibangun-dari-langkah-kaki</t>
+        </is>
+      </c>
+      <c r="H1163" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/pedesterian-deck-dukuh-atas-1786031934340_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1163" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Batu Bara Hasil Sitaan Laku Dilelang Rp 20,97 Miliar</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:29:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1164" t="inlineStr">
+        <is>
+          <t>Retno Ayuningrum</t>
+        </is>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>Kementerian ESDM menyampaikan PNBP hasil lelang Barang yang Dikuasai Negara berupa batu bara hasil penegakan hukum di Kalimantan Timur sebesar Rp 20,97 miliar.</t>
+        </is>
+      </c>
+      <c r="F1164" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1164" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8607752/batu-bara-hasil-sitaan-laku-dilelang-rp-20-97-miliar</t>
+        </is>
+      </c>
+      <c r="H1164" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/batu-bara-hasil-penindakan-hukum-laku-dilelang-1786030053576_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1164" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Wajah Musdalifah Basri Iritasi Akibat Totalitas saat Bikin Konten</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:09:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1165" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E1165" t="inlineStr">
+        <is>
+          <t>Komika Musdalifah Basri berbagi pengalaman buruk setelah menggunakan pewarna wajah berbahaya untuk konten. Kini, ia lebih berhati-hati dalam berkreasi.</t>
+        </is>
+      </c>
+      <c r="F1165" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1165" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8606916/wajah-musdalifah-basri-iritasi-akibat-totalitas-saat-bikin-konten</t>
+        </is>
+      </c>
+      <c r="H1165" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/musdalifah-basri-1786000069978_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1165" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Klarifikasi Sarwendah Minta Tambah Tiket Konser BLACKPINK kepada Ruben Onsu</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:01:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1166" t="inlineStr">
+        <is>
+          <t>Muhammad Ahsan Nurrijal</t>
+        </is>
+      </c>
+      <c r="E1166" t="inlineStr">
+        <is>
+          <t>Permintaan Sarwendah tambah tiket konser BLACKPINK jadi salah satu pemicu masalah dengan Ruben Onsu. Pihak Sarwendah klarifikasi soal ini.</t>
+        </is>
+      </c>
+      <c r="F1166" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1166" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8607627/klarifikasi-sarwendah-minta-tambah-tiket-konser-blackpink-kepada-ruben-onsu</t>
+        </is>
+      </c>
+      <c r="H1166" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/ruben-onsu-dan-sarwendah-1785990958073_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1166" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>Hot</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>MUA Bubah Alfian Cerita Detik Menegangkan Kecelakaan Mobil</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:25:09 +0700</t>
+        </is>
+      </c>
+      <c r="D1167" t="inlineStr">
+        <is>
+          <t>Febryantino Nur Pratama</t>
+        </is>
+      </c>
+      <c r="E1167" t="inlineStr">
+        <is>
+          <t>Makeup Artist Bubah Alfian menceritakan kecelakaan mobil setelah Jember Fashion Carnaval. Kelelahan dan kecepatan diduga jadi penyebab utama insiden tersebut.</t>
+        </is>
+      </c>
+      <c r="F1167" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1167" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8606994/mua-bubah-alfian-cerita-detik-menegangkan-kecelakaan-mobil</t>
+        </is>
+      </c>
+      <c r="H1167" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/08/06/bubah-alfian-1785990698424_43.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1167" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Trump Serang Kandidat Senat Muslim Michigan: Dia Penuh Omong Kosong</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:30:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1168" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1168" t="inlineStr">
+        <is>
+          <t>Presiden Amerika Serikat menyerang kandidat Senat Michigan, Abdul El-Sayed yang merupakan seorang Muslim pada Rabu (5/8).</t>
+        </is>
+      </c>
+      <c r="F1168" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1168" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260806121802-139-1389244/trump-serang-kandidat-senat-muslim-michigan-dia-penuh-omong-kosong</t>
+        </is>
+      </c>
+      <c r="H1168" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/thumbnail-video-1785993732321_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1168" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>JD Vance Akui Negosiasi dengan Israel Amat Sulit</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:56:30 +0700</t>
+        </is>
+      </c>
+      <c r="D1169" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1169" t="inlineStr">
+        <is>
+          <t>Wakil Presiden Amerika Serikat JD Vance mengakui pembicaraan dengan Iran amat sulit.</t>
+        </is>
+      </c>
+      <c r="F1169" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1169" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260806201629-134-1389493/jd-vance-akui-negosiasi-dengan-israel-amat-sulit</t>
+        </is>
+      </c>
+      <c r="H1169" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/04/11/wapres-as-jd-vance-1775872516501_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1169" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>Internasional</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Pelobi Israel 'Siram' Rp536 M Demi Jegal Kandidat AS Pro Palestina</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:18:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1170" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1170" t="inlineStr">
+        <is>
+          <t>Kelompok pelobi pro Israel yang sudah aktif sejak tahun 1950-an ini, disebut telah menggelontorkan dana hingga setara kurang lebih Rp536 miliar.</t>
+        </is>
+      </c>
+      <c r="F1170" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1170" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/internasional/20260806200347-134-1389490/pelobi-israel-siram-rp536-m-demi-jegal-kandidat-as-pro-palestina</t>
+        </is>
+      </c>
+      <c r="H1170" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/05/07/menlu-as-antony-blinken-beri-sambutan-di-acara-aipac_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1170" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Bank-Bank Diminta Siaga Hadapi Petaka Besar, Korbannya Sudah Banyak</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:00:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1171" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1171" t="inlineStr">
+        <is>
+          <t>Teknologi AI canggih membawa ancaman serius, dengan insiden pembobolan perusahaan. JPMorgan pimpin aliansi untuk mitigasi risiko.</t>
+        </is>
+      </c>
+      <c r="F1171" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1171" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260806124358-37-757098/bank-bank-diminta-siaga-hadapi-petaka-besar-korbannya-sudah-banyak</t>
+        </is>
+      </c>
+      <c r="H1171" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/07/21/jp-morgan-chase-1784617169554_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1171" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Bunga di China Ternyata Makan Daging, Bentuknya Mengejutkan</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1172" t="inlineStr">
+        <is>
+          <t>Redaksi</t>
+        </is>
+      </c>
+      <c r="E1172" t="inlineStr">
+        <is>
+          <t>Penemuan mengejutkan, bunga liar Saxifraga candelabrum di China barat daya adalah tumbuhan karnivora pertama di genusnya.</t>
+        </is>
+      </c>
+      <c r="F1172" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1172" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260806061231-37-757111/bunga-di-china-ternyata-makan-daging-bentuknya-mengejutkan</t>
+        </is>
+      </c>
+      <c r="H1172" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/08/06/rambut-kelenjar-yang-lengket-pada-spesies-tanaman-saxifraga-candelabrum-terlihat-sedang-memerangkap-serangga-mangsa-dalam-foto-1785997193512_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1172" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Ternyata Monyet Punya Binatang Peliharaan Seperti Manusia</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:40:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1173" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1173" t="inlineStr">
+        <is>
+          <t>Penelitian Universitas Oxford mengungkap kera dan monyet juga merawat hewan dari spesies berbeda.</t>
+        </is>
+      </c>
+      <c r="F1173" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1173" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260806134904-37-757131/ternyata-monyet-punya-binatang-peliharaan-seperti-manusia</t>
+        </is>
+      </c>
+      <c r="H1173" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2026/02/20/seekor-bayi-monyet-bernama-punch-menjadi-pusat-perhatian-di-media-sosial-punch-merupakan-bayi-monyet-di-kebun-binatang-ichikaw-1771567865691_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1173" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Raja Ojol Tutup di RI, Sekarang Menggila Ancam Driver Online</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1174" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1174" t="inlineStr">
+        <is>
+          <t>Uber siapkan lebih dari Rp180 triliun untuk ekspansi taksi robot tanpa sopir. Simak selengkapnya!</t>
+        </is>
+      </c>
+      <c r="F1174" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1174" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260806162635-37-757195/raja-ojol-tutup-di-ri-sekarang-menggila-ancam-driver-online</t>
+        </is>
+      </c>
+      <c r="H1174" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2018/01/26/9d2fddd0-0e40-4370-a7f5-57170fa82b49_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1174" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>Tech</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Perusahaan China Bangkrut, Bos Besar Langsung Dihukum Mati</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 18:20:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1175" t="inlineStr">
+        <is>
+          <t>Intan Rakhmayanti</t>
+        </is>
+      </c>
+      <c r="E1175" t="inlineStr">
+        <is>
+          <t>Pengadilan China menjatuhkan hukuman mati kepada Zhao Weiguo, mantan Komisaris Utama Tsinghua Unigroup.</t>
+        </is>
+      </c>
+      <c r="F1175" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1175" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/tech/20260806162050-37-757192/perusahaan-china-bangkrut-bos-besar-langsung-dihukum-mati</t>
+        </is>
+      </c>
+      <c r="H1175" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/05/15/ketua-tsinghua-unigroup-zhao-weiguo-terlihat-selama-wawancara-dengan-reuters-di-beijing-tiongkok-15-november-2015-1747293725188_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1175" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>Finansial</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Said: Ekonomi Tumbuh 5,29 Persen Patut Disyukuri, Tapi Industri dan Pertanian Harus Diwaspadai</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:35:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1176" t="inlineStr">
+        <is>
+          <t>Nashih Nashrullah</t>
+        </is>
+      </c>
+      <c r="E1176" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA — Ketua Badan Anggaran (Banggar) DPR RI Said Abdullah mengapresiasi capaian pertumbuhan ekonomi Indonesia yang mencapai 5,29 persen secara tahunan (year on year/yoy) pada triwulan II 2026, di...</t>
+        </is>
+      </c>
+      <c r="F1176" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1176" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjcezx320/said-ekonomi-tumbuh-529-persen-patut-disyukuri-tapi-industri-dan-pertanian-harus-diwaspadai</t>
+        </is>
+      </c>
+      <c r="H1176" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/ketua-dpp-pdip-yang-juga-ketua-badan-anggaran-banggar_220906182440-582.jpg</t>
+        </is>
+      </c>
+      <c r="I1176" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>Bisnis</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>NCC 2026 Dorong Kolaborasi Perkuat Keamanan Siber dan Ekonomi Digital</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:48:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1177" t="inlineStr">
+        <is>
+          <t>Friska Yolandha</t>
+        </is>
+      </c>
+      <c r="E1177" t="inlineStr">
+        <is>
+          <t>REPUBLIKA.CO.ID, JAKARTA — Penguatan keamanan siber dinilai menjadi prasyarat utama untuk menjaga laju pertumbuhan ekonomi digital Indonesia di tengah semakin masifnya adopsi kecerdasan buatan (artificial intelligence/AI). Tanpa sistem keamanan...</t>
+        </is>
+      </c>
+      <c r="F1177" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1177" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/tjcmg2370/ncc-2026-dorong-kolaborasi-perkuat-keamanan-siber-dan-ekonomi-digital</t>
+        </is>
+      </c>
+      <c r="H1177" t="inlineStr">
+        <is>
+          <t>https://static.republika.co.id/uploads/images/detailnews/_260806195140-854.png</t>
+        </is>
+      </c>
+      <c r="I1177" t="inlineStr">
+        <is>
+          <t>Republika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Siasat Agar Tak Antre di SPBU Berjam-jam</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:03:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1178" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1178" t="inlineStr">
+        <is>
+          <t>Antrean panjang di SPBU membuat pengendara menyusun strategi. Ada yang rela mengisi bensin tengah malam, sementara yang lain memilih membayar lebih mahal demi menghemat waktu.</t>
+        </is>
+      </c>
+      <c r="F1178" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1178" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8263527/siasat-agar-tak-antre-di-spbu-berjam-jam</t>
+        </is>
+      </c>
+      <c r="H1178" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/B5vF_oqPo37pI7NMT6YfNm-drvQ=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317227/original/083215400_1786007013-IMG_20260806_100057_766.jpg</t>
+        </is>
+      </c>
+      <c r="I1178" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Detik-Detik 2 Remaja Nyambi Kurir Sabu Tak Berkutik saat Dibekuk</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 23:06:36 +0700</t>
+        </is>
+      </c>
+      <c r="D1179" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1179" t="inlineStr">
+        <is>
+          <t>Keduanya sempat dikepung warga.</t>
+        </is>
+      </c>
+      <c r="F1179" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1179" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8263876/detik-detik-2-remaja-nyambi-kurir-sabu-tak-berkutik-saat-dibekuk</t>
+        </is>
+      </c>
+      <c r="H1179" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/FgsrshL7R0LyFPttCAwrj8fdd8k=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317637/original/064591800_1786032367-IMG-20260806-WA0019.jpg</t>
+        </is>
+      </c>
+      <c r="I1179" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Eks Ketua DPRD Ponorogo Jadi Tersangka Dugaan Korupsi Tunjangan Perumahan</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:55:12 +0700</t>
+        </is>
+      </c>
+      <c r="D1180" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1180" t="inlineStr">
+        <is>
+          <t>SN kini ditahan di Rumah Tahanan Kelas IIB Ponorogo selama 20 hari untuk kepentingan penyidikan.</t>
+        </is>
+      </c>
+      <c r="F1180" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1180" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8263871/eks-ketua-dprd-ponorogo-jadi-tersangka-dugaan-korupsi-tunjangan-perumahan</t>
+        </is>
+      </c>
+      <c r="H1180" t="inlineStr">
+        <is>
+          <t>https://cdn1-production-images-kly.akamaized.net/iqwEsRApikkILHu3rLmVdAtxFKI=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317631/original/047526200_1786031385-462812.jpg</t>
+        </is>
+      </c>
+      <c r="I1180" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Kasus Mutilasi di Depok, Pelaku Resign dari Tempat Kerja Saat Hari Kejadian</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:21:44 +0700</t>
+        </is>
+      </c>
+      <c r="D1181" t="inlineStr">
+        <is>
+          <t>Redaksi Liputan6</t>
+        </is>
+      </c>
+      <c r="E1181" t="inlineStr">
+        <is>
+          <t>Sehari sebelum peristiwa pembunuhan, pelaku minta libur dengan alasan mengikuti wawancara kerja di sebuah food court mal.</t>
+        </is>
+      </c>
+      <c r="F1181" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1181" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8263859/kasus-mutilasi-di-depok-pelaku-resign-dari-tempat-kerja-saat-hari-kejadian</t>
+        </is>
+      </c>
+      <c r="H1181" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/jk0mg0oz_NYTomVposjWMV7bOa4=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/9317152/original/097817700_1786004215-email-attachment_2026_08_06_dicky-agung-prihanto_polisi-lakukan-pencarian-potongan-tubuh-korban-mutilasi-disepanjang-kali-licin-depok_IMG-20260806-WA0016.jpg</t>
+        </is>
+      </c>
+      <c r="I1181" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1138"/>
+  <autoFilter ref="A1:I1181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 02:04 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1181"/>
+  <dimension ref="A1:I1182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -55945,8 +55945,55 @@
         </is>
       </c>
     </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Lima Klaster Budidaya Rumput Laut, Mesin Penggerak Ekonomi Pesisir NTT</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 16:43:28 +0700</t>
+        </is>
+      </c>
+      <c r="D1182" t="inlineStr">
+        <is>
+          <t>Liputan6.com</t>
+        </is>
+      </c>
+      <c r="E1182" t="inlineStr">
+        <is>
+          <t>Pemprov NTT menyiapkan lima klaster budidaya rumput laut  untuk memperkuat ekonomi pesisir melalui industri rumput laut yang terintegrasi dari hulu hingga hilir.</t>
+        </is>
+      </c>
+      <c r="F1182" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1182" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/8258000/lima-klaster-budidaya-rumput-laut-mesin-penggerak-ekonomi-pesisir-ntt</t>
+        </is>
+      </c>
+      <c r="H1182" t="inlineStr">
+        <is>
+          <t>https://cdn0-production-images-kly.akamaized.net/BEMmzSbMbghDJkycArhbEohHXRE=/673x379/smart/filters:quality(75):strip_icc():format(webp)/kly-media-production/medias/557605/original/100505bfoto_petani-laut.jpg</t>
+        </is>
+      </c>
+      <c r="I1182" t="inlineStr">
+        <is>
+          <t>Liputan6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1181"/>
+  <autoFilter ref="A1:I1182"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 08:09 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1310</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1311</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1310"/>
+  <dimension ref="A1:I1311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -62008,8 +62008,55 @@
         </is>
       </c>
     </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>Buruh Tetap Kawal Pembahasan RUU Ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 13:28:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>Ignacio Geordi Oswaldo</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Buruh menegaskan tetap berada dalam status siaga untuk mengawal pembahasan Rancangan Undang-Undang (RUU) Ketenagakerjaan di DPR RI.</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1311" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8606831/buruh-tetap-kawal-pembahasan-ruu-ketenagakerjaan</t>
+        </is>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/community/media/visual/2026/05/01/ilustrasi-kepadatan-lalin-saat-demo-buruh-1777601372612_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1311" t="inlineStr">
+        <is>
+          <t>Detik</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1310"/>
+  <autoFilter ref="A1:I1311"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 09:53 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1311</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1337</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1311"/>
+  <dimension ref="A1:I1337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -62055,8 +62055,1230 @@
         </is>
       </c>
     </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Menkum Tunggu DPR soal Penggantian Nama RUU Perampasan Aset</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:55:31 +0700</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>Menkum Supratman menunggu kabar DPR tentang usulan penggantian nama RUU Perampasan Aset. RUU ini sudah masuk prolegnas dan mendapat masukan dari para ahli.</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806213936-12-1389511/menkum-tunggu-dpr-soal-penggantian-nama-ruu-perampasan-aset</t>
+        </is>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/06/09/dpr-setujui-ruu-polri-jadi-undang-undang-1780995987689_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1312" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Prabowo: Investasi RnD Indonesia Masih Sedikit, Kita Perbaiki</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:50:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto mengakui rendahnya investasi RnD di Indonesia dan berkomitmen untuk meningkatkannya. Ia menekankan pentingnya kualitas pendidikan.</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1313" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806192627-20-1389473/prabowo-investasi-rnd-indonesia-masih-sedikit-kita-perbaiki</t>
+        </is>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/presiden-undang-150-periset-dan-peneliti-brin-ke-istana-1786016567897_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1313" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>Keluarga Korban KMP Mutiara Sentosa yang Masih Hilang Diminta Melapor</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:45:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr">
+        <is>
+          <t>Keluarga korban KMP Mutiara Sentosa II yang hilang diminta melapor ke Polres Tanjung Perak atau KSOP untuk mendukung proses pencarian oleh Basarnas.</t>
+        </is>
+      </c>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806204344-20-1389507/keluarga-korban-kmp-mutiara-sentosa-yang-masih-hilang-diminta-melapor</t>
+        </is>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/04/62-korban-kmp-mutiara-sentosa-ii-tiba-di-surabaya-dari-masalembu-1785831912067_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1314" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Polresta: Bripda RF Diduga Rencanakan Pembunuhan Lansia Deli Serdang</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:30:16 +0700</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr">
+        <is>
+          <t>Bripda RF ditetapkan sebagai tersangka pembunuhan berencana nenek Nurlis di Deliserdang. Tersangka merusak CCTV sebelum kejadian dan melarikan diri setelahnya.</t>
+        </is>
+      </c>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1315" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806201531-20-1389492/polresta-bripda-rf-diduga-rencanakan-pembunuhan-lansia-deli-serdang</t>
+        </is>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/09/14/5cf965a3-c769-46ef-a4b8-ca0c095cfd58_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1315" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>Pakar Hukum soal RUU Perampasan Aset: Lebih Tepat Istilah Pemulihan</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:18:20 +0700</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>Guru Besar Hukum Unissula usulkan istilah 'pemulihan aset' dalam RUU Perampasan Aset agar lebih restoratif.</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806203332-12-1389505/pakar-hukum-soal-ruu-perampasan-aset-lebih-tepat-istilah-pemulihan</t>
+        </is>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2019/10/31/57bd5113-e11c-46b7-948b-d8a96adbc8eb_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1316" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Menkum Bakal Gratiskan Tarif PNBP Pemberitahuan Laporan Tahunan RUPS</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:11:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>Menteri Hukum Supratman Agtas mengaku sedang mengusulkan ke Menkeu untuk penggratisan tarif PNBP pada laporan tahunan RUPS.</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806215103-20-1389512/menkum-bakal-gratiskan-tarif-pnbp-pemberitahuan-laporan-tahunan-rups</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/11/18/dpr-setujui-ruu-kuhap-menjadi-undang-undang-1763445439624_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1317" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>1 Tahun Kasus Dana CSR BI dan OJK, KPK Belum Tahan 2 Anggota DPR</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 22:07:23 +0700</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>KPK terus menyelidiki kasus korupsi dan pencucian uang terkait program sosial di BI dan OJK. Dua anggota DPR telah ditetapkan sebagai tersangka.</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806204652-12-1389508/1-tahun-kasus-dana-csr-bi-ojk-kpk-belum-tahan-2-anggota-dpr</t>
+        </is>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/03/05/ilustrasi-gedung-kpk-7_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1318" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>Korupsi Pesawat Fiktif, Eks Pegawai BUMN Tersangka Kejari Tangerang</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:58:58 +0700</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>Kejari Tangerang menetapkan FA, eks VP PT Angkasa Pura Cargo, sebagai tersangka korupsi pesawat fiktif. Proyek gagal, penyidikan masih berlanjut.</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1319" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260805105021-12-1388801/korupsi-pesawat-fiktif-eks-pegawai-bumn-tersangka-kejari-tangerang</t>
+        </is>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2021/09/08/ilustrasi-tindakan-kriminal-3_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1319" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>Tragedi Kebakaran Maut di Bombana Sultra, Ibu dan 4 Anak Tewas</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:45:29 +0700</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Kebakaran di Bombana, Sulawesi Tenggara, mengakibatkan tewasnya seorang ibu dan empat anak.</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1320" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806194611-20-1389489/tragedi-kebakaran-maut-di-bombana-sultra-ibu-dan-4-anak-tewas</t>
+        </is>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/12/24/ilustrasi-kebakaran-pabrik_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1320" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Usai Don Ritto, Tim 9 Kejagung Juga Geledah Rumah Nurman Herin</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:17:01 +0700</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Kejaksaan Agung menggeledah rumah Nurman Herin di Bandung terkait kasus TPPU emas 74 kg dan Rp543 miliar.</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806202827-12-1389504/usai-don-ritto-tim-9-kejagung-juga-geledah-rumah-nurman-herin</t>
+        </is>
+      </c>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/31/kejagung-tahan-nurman-herin-terkait-kasus-tppu-mantan-jampidsus-1785471654529_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1321" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>Usai Imbauan Walkot, Pengelola Mal Surabaya Kini Pendekkan Pagar</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:16:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Pengelola mal di Surabaya, Pakuwon Group, memendekkan pagar di Tunjungan Plaza dan Pakuwon Mall untuk menjaga estetika kota, sesuai imbauan Walkot Eri Cahyadi.</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806202621-20-1389503/usai-imbauan-walkot-pengelola-mal-surabaya-kini-pendekkan-pagar</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/usai-tinggikan-pengelola-mal-surabaya-kini-pendekkan-pagar-karena-imbauan-walkot-1786019976304_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1322" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>FOTO: Kebakaran Hutan Gunung Bromo, Kemenhut Kerahkan Operasi Terpadu</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:09:15 +0700</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan dan lahan seluas 70 hektare melanda Gunung Bromo hingga Kamis (6/8). Akibatnya, tiga akses masuk wisata kawasan Gunung Bromo.</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806190958-22-1389459/foto-kebakaran-hutan-gunung-bromo-kemenhut-kerahkan-operasi-terpadu</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/kebakaran-hutan-kawasan-gunung-bromo-1786018084811_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1323" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>FOTO: Karhutla dan Kekeringan Landa Boyolali Imbas Kemarau</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 21:00:40 +0700</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan dan lahan (karhutla) serta kekeringan melanda wilayah Boyolali, Jawa Tengah.</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806070138-22-1389129/foto-karhutla-dan-kekeringan-landa-boyolali-imbas-kemarau</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/pemadaman-kebakaran-kawasan-hutan-di-boyolali-1785974493169_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1324" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>KPK Lakukan Penggeledahan di Kota Bengkulu</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:40:27 +0700</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>KPK menggeledah lokasi di Kota Bengkulu terkait dugaan korupsi suap pengelolaan limbah kesehatan.</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806202244-12-1389495/kpk-lakukan-penggeledahan-di-kota-bengkulu</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2024/03/05/ilustrasi-gedung-kpk-8_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1325" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Pemilik soal Ratusan Airsoft Gun di Sekolah Jaksel: Buat Ekskul Nembak</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:36:49 +0700</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Direktur Utama PT Lokta Karya Perbakin menjelaskan bahwa 995 senjata airsoft yang ditemukan di sekolah Jaksel untuk ekstrakurikuler menembak.</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806200454-12-1389491/pemilik-soal-ratusan-airsoft-gun-di-sekolah-jaksel-buat-ekskul-nembak</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308099_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1326" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>TNI AD soal Wacana Sertifikat Pramuka Garuda Tanpa Tes: Tetap Seleksi</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:16:53 +0700</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>TNI AD menegaskan sertifikat Pramuka Garuda tidak menjamin penerimaan tanpa seleksi.</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806194631-12-1389477/tni-ad-soal-wacana-sertifikat-pramuka-garuda-tanpa-tes-tetap-seleksi</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2025/08/06/pengibaran-serentak-bendera-merah-putih-1754479814794_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1327" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Mangkir Lagi, KPK Ingatkan Rudy Tanoe Kooperatif</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:11:32 +0700</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>KPK mengingatkan Rudy Tanoe untuk kooperatif setelah mangkir dari panggilan. Dia penting dalam kasus dugaan korupsi bansos beras 2020.</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806194924-12-1389478/mangkir-lagi-kpk-ingatkan-rudy-tanoe-kooperatif</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2023/12/14/bambang-rudijanto-tanoesoedibjo_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1328" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Buntut Penebangan Pohon, Videotron di Padel Cihapit Bandung Disegel</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:05:43 +0700</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>Satpol PP Bandung segel videotron di SixNine Padel setelah penebangan 10 pohon tanpa izin. Penyelidikan masih berlanjut untuk mengungkap pihak terlibat.</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1329" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806144153-20-1389332/buntut-penebangan-pohon-videotron-di-padel-cihapit-bandung-disegel</t>
+        </is>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/penyegelan-videotron-sixnine-padel-buntut-penebangan-10-pohon-secara-ilegal-di-bandung-1786001631954_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1329" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Prabowo Tes Langsung Kekuatan Genteng Buatan BRIN</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:31:06 +0700</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto uji coba ketahanan genteng inovasi BRIN berbahan sabut kelapa. Kunjungan ini melibatkan 150 peneliti yang memamerkan temuan mereka.</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806183730-20-1389439/prabowo-tes-langsung-kekuatan-genteng-buatan-brin</t>
+        </is>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/presiden-undang-150-periset-dan-peneliti-brin-ke-istana-1786016568023_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1330" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>Pihak Sekolah di Jaksel Ungkap Momen Temukan Ratusan Senpi</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:23:04 +0700</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr">
+        <is>
+          <t>Kuasa hukum mengungkap 995 senjata ditemukan di ruang mantan ketua yayasan sekolah di Jakarta Selatan. Temuan ini termasuk senjata api dan narkoba.</t>
+        </is>
+      </c>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806184026-12-1389443/pihak-sekolah-di-jaksel-ungkap-momen-temukan-ratusan-senpi</t>
+        </is>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308099_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1331" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>Hasan Nasbi Duga Makalah MBG untuk Nobel Bukan dari Pemerintah</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:13:39 +0700</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Penasihat Presiden Prabowo buka suara soal makalah program Makan Bergizi Gratis yang diajukan jadi Nobel Perdamaian 2026.</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806185935-32-1389450/hasan-nasbi-duga-makalah-mbg-untuk-nobel-bukan-dari-pemerintah</t>
+        </is>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/04/27/hasan-nasbi-1777279292814_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1332" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>Selain Senpi, CD Porno-Narkoba Juga Ditemukan di Yayasan di Jaksel</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:10:18 +0700</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr">
+        <is>
+          <t>Ratusan senjata api, narkoba, dan CD porno diduga ditemukan di ruangan mantan ketua yayasan sekolah di Pondok Pinang, Jakarta Selatan</t>
+        </is>
+      </c>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806181924-12-1389432/selain-senpi-cd-porno-narkoba-juga-ditemukan-di-yayasan-di-jaksel</t>
+        </is>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1333" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>Dukung MBG di Wilayah 3T, Mendagri Siap Kerahkan Ditjen Dukcapil</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:05:07 +0700</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>Kemendagri</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr">
+        <is>
+          <t>Menurut Mendagri, masyarakat di wilayah 3T seperti Papua, NTT, dan Malukumerupakan kelompok yang paling membutuhkan perhatian pemerintah.</t>
+        </is>
+      </c>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806184637-25-1389444/dukung-mbg-di-wilayah-3t-mendagri-siap-kerahkan-ditjen-dukcapil</t>
+        </is>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/kemendagri-1786016909695_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1334" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Selain Senpi, Ada Ruang Diduga Bunker di Yayasan Sekolah Pondok Pinang</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 19:04:50 +0700</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Selain 995 senjata api, alat pembuat peluru, dan narkoba, gedung yayasan sekolah di Pondok Pinang Jaksel juga ditemukan ruang diduga bunker.</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806183504-12-1389448/selain-senpi-ada-ruang-diduga-bunker-di-yayasan-sekolah-pondok-pinang</t>
+        </is>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/08/06/995-senjata-yang-ditemukan-di-ruang-mantan-ketua-yayasan-sekolah-jaksel-1786011308187_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1335" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>Menkes Sedih Respons Banyak Nakes Cibir Pasien BPJS di Medsos</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 18:34:00 +0700</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr">
+        <is>
+          <t>Menkes Budi Gunadi Sadikin menanggapi komentar menghina pasien BPJS oleh tenaga kesehatan. Ia menekankan pentingnya empati dalam profesi kesehatan.</t>
+        </is>
+      </c>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1336" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806174644-20-1389415/menkes-sedih-respons-banyak-nakes-cibir-pasien-bpjs-di-medsos</t>
+        </is>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/01/07/pemerintah-pulihkan-pelayanan-kesehatan-di-wilayah-terdampak-bencana-1767781411341_169.jpeg?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1336" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>Nasional</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>Prabowo Antusias Cermati Perkembangan Teknologi dan Hasil Riset BRIN</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 18:05:48 +0700</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>Redaksi CNN Indonesia</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Presiden Prabowo Subianto mengunjungi pameran riset BRIN di Istana, melihat inovasi untuk program prioritas seperti ketahanan pangan dan energi.</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>https://www.cnnindonesia.com/nasional/20260806175333-20-1389418/prabowo-antusias-cermati-perkembangan-teknologi-dan-hasil-riset-brin</t>
+        </is>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>https://akcdn.detik.net.id/visual/2026/07/31/pertemuan-presiden-prabowo-dengan-pengusaha-kadin-1785486310599_169.png?w=360&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1337" t="inlineStr">
+        <is>
+          <t>CNN Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1311"/>
+  <autoFilter ref="A1:I1337"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update berita 2026-08-07 10:50 UTC
</commit_message>
<xml_diff>
--- a/data/berita_2026-08-06.xlsx
+++ b/data/berita_2026-08-06.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Berita" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1337</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Berita'!$A$1:$I$1338</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1337"/>
+  <dimension ref="A1:I1338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -63277,8 +63277,55 @@
         </is>
       </c>
     </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>News</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>Smelter Raksasa Bahan Baku Baterai EV Mulai Beroperasi di Sultra!</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 20:50:03 +0700</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>Redaksi CNBC Indonesia</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>PT Vale Indonesia Tbk menjadwalkan operasional atau startup proyek High Pressure Acid Leaching (HPAL) raksasa di Sulawesi Tenggara</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>Netral</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>https://www.cnbcindonesia.com/news/20260806175304-4-757242/smelter-raksasa-bahan-baku-baterai-ev-mulai-beroperasi-di-sultra</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>https://awsimages.detik.net.id/visual/2025/01/29/vale-reuterswashington-alvesfile-photo_169.jpeg?w=1200&amp;q=90</t>
+        </is>
+      </c>
+      <c r="I1338" t="inlineStr">
+        <is>
+          <t>CNBC Indonesia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I1337"/>
+  <autoFilter ref="A1:I1338"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>